<commit_message>
Ajout du fichier classeur
</commit_message>
<xml_diff>
--- a/POINTAGE_BRUT_AOUT_24.xlsx
+++ b/POINTAGE_BRUT_AOUT_24.xlsx
@@ -5,21 +5,24 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B.NIMI\Desktop\DIVERS\Emiles\HS_A_ANALYSER_AOUT26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B.NIMI\Desktop\DIVERS\Fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB71B60-6075-4388-B0D1-A745921401E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052224FB-FB7D-4C16-8FDF-6A7FB3FB2B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="POINTAGES" sheetId="1" r:id="rId1"/>
     <sheet name="HS" sheetId="3" r:id="rId2"/>
     <sheet name="CODE_POINTAGE" sheetId="2" r:id="rId3"/>
     <sheet name="Feuil1" sheetId="4" r:id="rId4"/>
+    <sheet name="Feuil2" sheetId="5" r:id="rId5"/>
+    <sheet name="Configurations" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Feuil1!$C$4:$K$35</definedName>
+    <definedName name="POSE_CSKN">Configurations!$K$5:$M$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="293">
   <si>
     <t>Matricule</t>
   </si>
@@ -885,6 +888,39 @@
   </si>
   <si>
     <t>66 sur 45 signifie 66 heures prestées / semaine sur 45 heures de prestation hebdomadaires fixés par le code du travail congolais par rapport aux nombre des h=jours prestés</t>
+  </si>
+  <si>
+    <t>Heures Prestées</t>
+  </si>
+  <si>
+    <t>Observation</t>
+  </si>
+  <si>
+    <t>Pas de présence physique</t>
+  </si>
+  <si>
+    <t>Présence physique</t>
+  </si>
+  <si>
+    <t>POINTAGE</t>
+  </si>
+  <si>
+    <t>POSE</t>
+  </si>
+  <si>
+    <t>HS Jr non ouvré</t>
+  </si>
+  <si>
+    <t>HS Jr  ouvré</t>
+  </si>
+  <si>
+    <t>Noel</t>
+  </si>
+  <si>
+    <t>Durée prestation</t>
+  </si>
+  <si>
+    <t>Férié</t>
   </si>
 </sst>
 </file>
@@ -894,7 +930,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00####"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -925,13 +961,19 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color theme="0"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -950,8 +992,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -974,11 +1022,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1063,12 +1168,177 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1079,6 +1349,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38945EDF-6FD5-4996-A655-EE0F60A9CF58}" name="Tableau_Pose_Cskn" displayName="Tableau_Pose_Cskn" ref="M2:N4" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+  <autoFilter ref="M2:N4" xr:uid="{38945EDF-6FD5-4996-A655-EE0F60A9CF58}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{FA25F88B-AD6F-4A5D-8F20-994C35E94325}" name="Date" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{BF59DA52-CD1D-4A0A-887A-22E32213672D}" name="Jour" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5981,10 +6265,10 @@
       <c r="E4" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="F4" s="25" t="s">
         <v>273</v>
       </c>
-      <c r="G4" s="34" t="s">
+      <c r="G4" s="25" t="s">
         <v>258</v>
       </c>
       <c r="J4" s="12" t="s">
@@ -6008,7 +6292,7 @@
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C5" s="23" t="str">
-        <f>TEXT(D5,"jjjj")</f>
+        <f t="shared" ref="C5:C35" si="0">TEXT(D5,"jjjj")</f>
         <v>dimanche</v>
       </c>
       <c r="D5" s="2">
@@ -6017,10 +6301,10 @@
       <c r="E5" s="1">
         <v>998</v>
       </c>
-      <c r="F5" s="34">
-        <v>12</v>
-      </c>
-      <c r="G5" s="34">
+      <c r="F5" s="25">
+        <v>12</v>
+      </c>
+      <c r="G5" s="25">
         <f>IF(F5-IF(C5="samedi",5,8)&lt;0,0,F5-IF(C5="samedi",5,8))</f>
         <v>4</v>
       </c>
@@ -6050,7 +6334,7 @@
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="str">
-        <f>TEXT(D6,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
       <c r="D6" s="2">
@@ -6059,11 +6343,11 @@
       <c r="E6" s="1">
         <v>997</v>
       </c>
-      <c r="F6" s="34">
+      <c r="F6" s="25">
         <v>18</v>
       </c>
-      <c r="G6" s="34">
-        <f t="shared" ref="G6:G35" si="0">IF(F6-IF(C6="samedi",5,8)&lt;0,0,F6-IF(C6="samedi",5,8))</f>
+      <c r="G6" s="25">
+        <f t="shared" ref="G6:G35" si="1">IF(F6-IF(C6="samedi",5,8)&lt;0,0,F6-IF(C6="samedi",5,8))</f>
         <v>10</v>
       </c>
       <c r="J6" s="22" t="s">
@@ -6079,7 +6363,7 @@
         <v>45495</v>
       </c>
       <c r="Q6" s="1" t="str">
-        <f t="shared" ref="Q6:Q35" si="1">TEXT(P6,"jjjj")</f>
+        <f t="shared" ref="Q6:Q35" si="2">TEXT(P6,"jjjj")</f>
         <v>lundi</v>
       </c>
       <c r="R6" s="1" t="s">
@@ -6092,7 +6376,7 @@
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C7" s="1" t="str">
-        <f>TEXT(D7,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
       <c r="D7" s="2">
@@ -6101,11 +6385,11 @@
       <c r="E7" s="1">
         <v>12</v>
       </c>
-      <c r="F7" s="34">
-        <v>0</v>
-      </c>
-      <c r="G7" s="34">
-        <f t="shared" si="0"/>
+      <c r="F7" s="25">
+        <v>0</v>
+      </c>
+      <c r="G7" s="25">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J7" s="22"/>
@@ -6117,7 +6401,7 @@
         <v>45496</v>
       </c>
       <c r="Q7" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mardi</v>
       </c>
       <c r="R7" s="1" t="s">
@@ -6130,7 +6414,7 @@
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C8" s="1" t="str">
-        <f>TEXT(D8,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
       <c r="D8" s="2">
@@ -6139,11 +6423,11 @@
       <c r="E8" s="1">
         <v>996</v>
       </c>
-      <c r="F8" s="34">
-        <v>12</v>
-      </c>
-      <c r="G8" s="34">
-        <f t="shared" si="0"/>
+      <c r="F8" s="25">
+        <v>12</v>
+      </c>
+      <c r="G8" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J8" s="22" t="s">
@@ -6159,7 +6443,7 @@
         <v>45497</v>
       </c>
       <c r="Q8" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mercredi</v>
       </c>
       <c r="R8" s="1" t="s">
@@ -6172,7 +6456,7 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C9" s="1" t="str">
-        <f>TEXT(D9,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
       <c r="D9" s="2">
@@ -6181,11 +6465,11 @@
       <c r="E9" s="1">
         <v>996</v>
       </c>
-      <c r="F9" s="34">
-        <v>12</v>
-      </c>
-      <c r="G9" s="34">
-        <f t="shared" si="0"/>
+      <c r="F9" s="25">
+        <v>12</v>
+      </c>
+      <c r="G9" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J9" s="22" t="s">
@@ -6201,7 +6485,7 @@
         <v>45498</v>
       </c>
       <c r="Q9" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>jeudi</v>
       </c>
       <c r="R9" s="1" t="s">
@@ -6214,7 +6498,7 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="str">
-        <f>TEXT(D10,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
       <c r="D10" s="2">
@@ -6223,11 +6507,11 @@
       <c r="E10" s="1">
         <v>996</v>
       </c>
-      <c r="F10" s="34">
-        <v>12</v>
-      </c>
-      <c r="G10" s="34">
-        <f t="shared" si="0"/>
+      <c r="F10" s="25">
+        <v>12</v>
+      </c>
+      <c r="G10" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J10" s="22" t="s">
@@ -6243,7 +6527,7 @@
         <v>45499</v>
       </c>
       <c r="Q10" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>vendredi</v>
       </c>
       <c r="R10" s="1" t="s">
@@ -6256,7 +6540,7 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C11" s="1" t="str">
-        <f>TEXT(D11,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
       <c r="D11" s="2">
@@ -6265,11 +6549,11 @@
       <c r="E11" s="1">
         <v>996</v>
       </c>
-      <c r="F11" s="34">
-        <v>12</v>
-      </c>
-      <c r="G11" s="34">
-        <f t="shared" si="0"/>
+      <c r="F11" s="25">
+        <v>12</v>
+      </c>
+      <c r="G11" s="25">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="J11" s="22" t="s">
@@ -6285,7 +6569,7 @@
         <v>45500</v>
       </c>
       <c r="Q11" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>samedi</v>
       </c>
       <c r="R11" s="1" t="s">
@@ -6298,7 +6582,7 @@
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C12" s="23" t="str">
-        <f>TEXT(D12,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
       <c r="D12" s="2">
@@ -6307,11 +6591,11 @@
       <c r="E12" s="1">
         <v>996</v>
       </c>
-      <c r="F12" s="34">
-        <v>12</v>
-      </c>
-      <c r="G12" s="34">
-        <f t="shared" si="0"/>
+      <c r="F12" s="25">
+        <v>12</v>
+      </c>
+      <c r="G12" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J12" s="22" t="s">
@@ -6327,7 +6611,7 @@
         <v>45501</v>
       </c>
       <c r="Q12" s="23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>dimanche</v>
       </c>
       <c r="R12" s="1" t="s">
@@ -6340,7 +6624,7 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="str">
-        <f>TEXT(D13,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
       <c r="D13" s="2">
@@ -6349,11 +6633,11 @@
       <c r="E13" s="1">
         <v>997</v>
       </c>
-      <c r="F13" s="34">
+      <c r="F13" s="25">
         <v>18</v>
       </c>
-      <c r="G13" s="34">
-        <f t="shared" si="0"/>
+      <c r="G13" s="25">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="J13" s="22" t="s">
@@ -6369,7 +6653,7 @@
         <v>45502</v>
       </c>
       <c r="Q13" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>lundi</v>
       </c>
       <c r="R13" s="1" t="s">
@@ -6382,7 +6666,7 @@
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="str">
-        <f>TEXT(D14,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
       <c r="D14" s="2">
@@ -6391,11 +6675,11 @@
       <c r="E14" s="1">
         <v>998</v>
       </c>
-      <c r="F14" s="34">
-        <v>12</v>
-      </c>
-      <c r="G14" s="34">
-        <f t="shared" si="0"/>
+      <c r="F14" s="25">
+        <v>12</v>
+      </c>
+      <c r="G14" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J14" s="22" t="s">
@@ -6411,7 +6695,7 @@
         <v>45503</v>
       </c>
       <c r="Q14" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mardi</v>
       </c>
       <c r="R14" s="1" t="s">
@@ -6424,7 +6708,7 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="str">
-        <f>TEXT(D15,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
       <c r="D15" s="2">
@@ -6433,11 +6717,11 @@
       <c r="E15" s="1">
         <v>998</v>
       </c>
-      <c r="F15" s="34">
-        <v>12</v>
-      </c>
-      <c r="G15" s="34">
-        <f t="shared" si="0"/>
+      <c r="F15" s="25">
+        <v>12</v>
+      </c>
+      <c r="G15" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J15" s="22" t="s">
@@ -6453,7 +6737,7 @@
         <v>45504</v>
       </c>
       <c r="Q15" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mercredi</v>
       </c>
       <c r="R15" s="1" t="s">
@@ -6466,7 +6750,7 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C16" s="23" t="str">
-        <f>TEXT(D16,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
       <c r="D16" s="2">
@@ -6475,11 +6759,11 @@
       <c r="E16" s="1">
         <v>998</v>
       </c>
-      <c r="F16" s="34">
-        <v>12</v>
-      </c>
-      <c r="G16" s="34">
-        <f t="shared" si="0"/>
+      <c r="F16" s="25">
+        <v>12</v>
+      </c>
+      <c r="G16" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J16" s="22" t="s">
@@ -6495,7 +6779,7 @@
         <v>45505</v>
       </c>
       <c r="Q16" s="23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>jeudi</v>
       </c>
       <c r="R16" s="1" t="s">
@@ -6508,7 +6792,7 @@
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C17" s="1" t="str">
-        <f>TEXT(D17,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
       <c r="D17" s="2">
@@ -6517,11 +6801,11 @@
       <c r="E17" s="1">
         <v>998</v>
       </c>
-      <c r="F17" s="34">
-        <v>12</v>
-      </c>
-      <c r="G17" s="34">
-        <f t="shared" si="0"/>
+      <c r="F17" s="25">
+        <v>12</v>
+      </c>
+      <c r="G17" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J17" s="22" t="s">
@@ -6537,7 +6821,7 @@
         <v>45506</v>
       </c>
       <c r="Q17" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>vendredi</v>
       </c>
       <c r="R17" s="1" t="s">
@@ -6548,7 +6832,7 @@
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C18" s="1" t="str">
-        <f>TEXT(D18,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
       <c r="D18" s="2">
@@ -6557,11 +6841,11 @@
       <c r="E18" s="1">
         <v>998</v>
       </c>
-      <c r="F18" s="34">
-        <v>12</v>
-      </c>
-      <c r="G18" s="34">
-        <f t="shared" si="0"/>
+      <c r="F18" s="25">
+        <v>12</v>
+      </c>
+      <c r="G18" s="25">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="J18" s="22" t="s">
@@ -6577,7 +6861,7 @@
         <v>45507</v>
       </c>
       <c r="Q18" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>samedi</v>
       </c>
       <c r="R18" s="1" t="s">
@@ -6590,7 +6874,7 @@
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C19" s="23" t="str">
-        <f>TEXT(D19,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
       <c r="D19" s="2">
@@ -6599,11 +6883,11 @@
       <c r="E19" s="1">
         <v>998</v>
       </c>
-      <c r="F19" s="34">
-        <v>12</v>
-      </c>
-      <c r="G19" s="34">
-        <f t="shared" si="0"/>
+      <c r="F19" s="25">
+        <v>12</v>
+      </c>
+      <c r="G19" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J19" s="22" t="s">
@@ -6619,7 +6903,7 @@
         <v>45508</v>
       </c>
       <c r="Q19" s="23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>dimanche</v>
       </c>
       <c r="R19" s="1" t="s">
@@ -6632,7 +6916,7 @@
     </row>
     <row r="20" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C20" s="1" t="str">
-        <f>TEXT(D20,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
       <c r="D20" s="2">
@@ -6641,11 +6925,11 @@
       <c r="E20" s="1">
         <v>997</v>
       </c>
-      <c r="F20" s="34">
+      <c r="F20" s="25">
         <v>18</v>
       </c>
-      <c r="G20" s="34">
-        <f t="shared" si="0"/>
+      <c r="G20" s="25">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="J20" s="22" t="s">
@@ -6661,7 +6945,7 @@
         <v>45509</v>
       </c>
       <c r="Q20" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>lundi</v>
       </c>
       <c r="R20" s="1" t="s">
@@ -6674,7 +6958,7 @@
     </row>
     <row r="21" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C21" s="1" t="str">
-        <f>TEXT(D21,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
       <c r="D21" s="2">
@@ -6683,11 +6967,11 @@
       <c r="E21" s="1">
         <v>12</v>
       </c>
-      <c r="F21" s="34">
-        <v>0</v>
-      </c>
-      <c r="G21" s="34">
-        <f t="shared" si="0"/>
+      <c r="F21" s="25">
+        <v>0</v>
+      </c>
+      <c r="G21" s="25">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J21" s="22"/>
@@ -6699,7 +6983,7 @@
         <v>45510</v>
       </c>
       <c r="Q21" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mardi</v>
       </c>
       <c r="R21" s="1" t="s">
@@ -6712,7 +6996,7 @@
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C22" s="1" t="str">
-        <f>TEXT(D22,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
       <c r="D22" s="2">
@@ -6721,11 +7005,11 @@
       <c r="E22" s="1">
         <v>996</v>
       </c>
-      <c r="F22" s="34">
-        <v>12</v>
-      </c>
-      <c r="G22" s="34">
-        <f t="shared" si="0"/>
+      <c r="F22" s="25">
+        <v>12</v>
+      </c>
+      <c r="G22" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J22" s="22" t="s">
@@ -6741,7 +7025,7 @@
         <v>45511</v>
       </c>
       <c r="Q22" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mercredi</v>
       </c>
       <c r="R22" s="1" t="s">
@@ -6754,7 +7038,7 @@
     </row>
     <row r="23" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C23" s="1" t="str">
-        <f>TEXT(D23,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
       <c r="D23" s="2">
@@ -6763,11 +7047,11 @@
       <c r="E23" s="1">
         <v>996</v>
       </c>
-      <c r="F23" s="34">
-        <v>12</v>
-      </c>
-      <c r="G23" s="34">
-        <f t="shared" si="0"/>
+      <c r="F23" s="25">
+        <v>12</v>
+      </c>
+      <c r="G23" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J23" s="22" t="s">
@@ -6783,7 +7067,7 @@
         <v>45512</v>
       </c>
       <c r="Q23" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>jeudi</v>
       </c>
       <c r="R23" s="1" t="s">
@@ -6796,7 +7080,7 @@
     </row>
     <row r="24" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C24" s="1" t="str">
-        <f>TEXT(D24,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
       <c r="D24" s="2">
@@ -6805,11 +7089,11 @@
       <c r="E24" s="1">
         <v>996</v>
       </c>
-      <c r="F24" s="34">
-        <v>12</v>
-      </c>
-      <c r="G24" s="34">
-        <f t="shared" si="0"/>
+      <c r="F24" s="25">
+        <v>12</v>
+      </c>
+      <c r="G24" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J24" s="22" t="s">
@@ -6825,7 +7109,7 @@
         <v>45513</v>
       </c>
       <c r="Q24" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>vendredi</v>
       </c>
       <c r="R24" s="1" t="s">
@@ -6838,7 +7122,7 @@
     </row>
     <row r="25" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C25" s="1" t="str">
-        <f>TEXT(D25,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
       <c r="D25" s="2">
@@ -6847,11 +7131,11 @@
       <c r="E25" s="1">
         <v>996</v>
       </c>
-      <c r="F25" s="34">
-        <v>12</v>
-      </c>
-      <c r="G25" s="34">
-        <f t="shared" si="0"/>
+      <c r="F25" s="25">
+        <v>12</v>
+      </c>
+      <c r="G25" s="25">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="J25" s="22" t="s">
@@ -6867,7 +7151,7 @@
         <v>45514</v>
       </c>
       <c r="Q25" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>samedi</v>
       </c>
       <c r="R25" s="1" t="s">
@@ -6880,7 +7164,7 @@
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C26" s="23" t="str">
-        <f>TEXT(D26,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
       <c r="D26" s="2">
@@ -6889,11 +7173,11 @@
       <c r="E26" s="1">
         <v>996</v>
       </c>
-      <c r="F26" s="34">
-        <v>12</v>
-      </c>
-      <c r="G26" s="34">
-        <f t="shared" si="0"/>
+      <c r="F26" s="25">
+        <v>12</v>
+      </c>
+      <c r="G26" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J26" s="22" t="s">
@@ -6909,7 +7193,7 @@
         <v>45515</v>
       </c>
       <c r="Q26" s="23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>dimanche</v>
       </c>
       <c r="R26" s="1" t="s">
@@ -6922,7 +7206,7 @@
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C27" s="1" t="str">
-        <f>TEXT(D27,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
       <c r="D27" s="2">
@@ -6931,11 +7215,11 @@
       <c r="E27" s="1">
         <v>997</v>
       </c>
-      <c r="F27" s="34">
+      <c r="F27" s="25">
         <v>18</v>
       </c>
-      <c r="G27" s="34">
-        <f t="shared" si="0"/>
+      <c r="G27" s="25">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="J27" s="22" t="s">
@@ -6951,7 +7235,7 @@
         <v>45516</v>
       </c>
       <c r="Q27" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>lundi</v>
       </c>
       <c r="R27" s="1" t="s">
@@ -6964,7 +7248,7 @@
     </row>
     <row r="28" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C28" s="1" t="str">
-        <f>TEXT(D28,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
       <c r="D28" s="2">
@@ -6973,11 +7257,11 @@
       <c r="E28" s="1">
         <v>998</v>
       </c>
-      <c r="F28" s="34">
-        <v>12</v>
-      </c>
-      <c r="G28" s="34">
-        <f t="shared" si="0"/>
+      <c r="F28" s="25">
+        <v>12</v>
+      </c>
+      <c r="G28" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J28" s="22" t="s">
@@ -6993,7 +7277,7 @@
         <v>45517</v>
       </c>
       <c r="Q28" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mardi</v>
       </c>
       <c r="R28" s="1" t="s">
@@ -7006,7 +7290,7 @@
     </row>
     <row r="29" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C29" s="1" t="str">
-        <f>TEXT(D29,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
       <c r="D29" s="2">
@@ -7015,11 +7299,11 @@
       <c r="E29" s="1">
         <v>998</v>
       </c>
-      <c r="F29" s="34">
-        <v>12</v>
-      </c>
-      <c r="G29" s="34">
-        <f t="shared" si="0"/>
+      <c r="F29" s="25">
+        <v>12</v>
+      </c>
+      <c r="G29" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J29" s="22" t="s">
@@ -7035,7 +7319,7 @@
         <v>45518</v>
       </c>
       <c r="Q29" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mercredi</v>
       </c>
       <c r="R29" s="1" t="s">
@@ -7048,7 +7332,7 @@
     </row>
     <row r="30" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C30" s="1" t="str">
-        <f>TEXT(D30,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
       <c r="D30" s="2">
@@ -7057,11 +7341,11 @@
       <c r="E30" s="1">
         <v>998</v>
       </c>
-      <c r="F30" s="34">
-        <v>12</v>
-      </c>
-      <c r="G30" s="34">
-        <f t="shared" si="0"/>
+      <c r="F30" s="25">
+        <v>12</v>
+      </c>
+      <c r="G30" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J30" s="22" t="s">
@@ -7077,7 +7361,7 @@
         <v>45519</v>
       </c>
       <c r="Q30" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>jeudi</v>
       </c>
       <c r="R30" s="1" t="s">
@@ -7090,7 +7374,7 @@
     </row>
     <row r="31" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C31" s="1" t="str">
-        <f>TEXT(D31,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
       <c r="D31" s="2">
@@ -7099,11 +7383,11 @@
       <c r="E31" s="1">
         <v>998</v>
       </c>
-      <c r="F31" s="34">
-        <v>12</v>
-      </c>
-      <c r="G31" s="34">
-        <f t="shared" si="0"/>
+      <c r="F31" s="25">
+        <v>12</v>
+      </c>
+      <c r="G31" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J31" s="22" t="s">
@@ -7119,7 +7403,7 @@
         <v>45520</v>
       </c>
       <c r="Q31" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>vendredi</v>
       </c>
       <c r="R31" s="1" t="s">
@@ -7132,7 +7416,7 @@
     </row>
     <row r="32" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="str">
-        <f>TEXT(D32,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
       <c r="D32" s="2">
@@ -7141,11 +7425,11 @@
       <c r="E32" s="1">
         <v>12</v>
       </c>
-      <c r="F32" s="34">
-        <v>0</v>
-      </c>
-      <c r="G32" s="34">
-        <f t="shared" si="0"/>
+      <c r="F32" s="25">
+        <v>0</v>
+      </c>
+      <c r="G32" s="25">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J32" s="22"/>
@@ -7157,7 +7441,7 @@
         <v>45521</v>
       </c>
       <c r="Q32" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>samedi</v>
       </c>
       <c r="R32" s="1" t="s">
@@ -7170,7 +7454,7 @@
     </row>
     <row r="33" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C33" s="23" t="str">
-        <f>TEXT(D33,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
       <c r="D33" s="2">
@@ -7179,11 +7463,11 @@
       <c r="E33" s="1">
         <v>998</v>
       </c>
-      <c r="F33" s="34">
-        <v>12</v>
-      </c>
-      <c r="G33" s="34">
-        <f t="shared" si="0"/>
+      <c r="F33" s="25">
+        <v>12</v>
+      </c>
+      <c r="G33" s="25">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="J33" s="22" t="s">
@@ -7199,7 +7483,7 @@
         <v>45522</v>
       </c>
       <c r="Q33" s="23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>dimanche</v>
       </c>
       <c r="R33" s="1" t="s">
@@ -7212,7 +7496,7 @@
     </row>
     <row r="34" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C34" s="1" t="str">
-        <f>TEXT(D34,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
       <c r="D34" s="2">
@@ -7221,11 +7505,11 @@
       <c r="E34" s="1">
         <v>997</v>
       </c>
-      <c r="F34" s="34">
+      <c r="F34" s="25">
         <v>18</v>
       </c>
-      <c r="G34" s="34">
-        <f t="shared" si="0"/>
+      <c r="G34" s="25">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="J34" s="22" t="s">
@@ -7241,7 +7525,7 @@
         <v>45523</v>
       </c>
       <c r="Q34" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>lundi</v>
       </c>
       <c r="R34" s="1" t="s">
@@ -7254,7 +7538,7 @@
     </row>
     <row r="35" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C35" s="1" t="str">
-        <f>TEXT(D35,"jjjj")</f>
+        <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
       <c r="D35" s="2">
@@ -7263,11 +7547,11 @@
       <c r="E35" s="1">
         <v>12</v>
       </c>
-      <c r="F35" s="34">
-        <v>0</v>
-      </c>
-      <c r="G35" s="34">
-        <f t="shared" si="0"/>
+      <c r="F35" s="25">
+        <v>0</v>
+      </c>
+      <c r="G35" s="25">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J35" s="22"/>
@@ -7279,7 +7563,7 @@
         <v>45524</v>
       </c>
       <c r="Q35" s="1" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>mardi</v>
       </c>
       <c r="R35" s="1" t="s">
@@ -7495,4 +7779,2985 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0091FD1A-61FC-47E9-AD25-A4EDDFCE69B5}">
+  <dimension ref="B2:N34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="8.7265625" customWidth="1"/>
+    <col min="5" max="5" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:14" ht="26" x14ac:dyDescent="0.3">
+      <c r="B2" s="41" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" s="41" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" s="42" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="51" t="s">
+        <v>291</v>
+      </c>
+      <c r="F2" s="44" t="s">
+        <v>289</v>
+      </c>
+      <c r="G2" s="44" t="s">
+        <v>288</v>
+      </c>
+      <c r="I2" s="25"/>
+      <c r="M2" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="N2" s="46" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B3" s="37" t="str">
+        <f t="shared" ref="B3:B33" si="0">TEXT(C3,"jjjj")</f>
+        <v>dimanche</v>
+      </c>
+      <c r="C3" s="38">
+        <v>45494</v>
+      </c>
+      <c r="D3" s="39">
+        <v>998</v>
+      </c>
+      <c r="E3" s="12">
+        <f>IF(LEN(TRIM(D3))=2,VLOOKUP(TEXT(D3,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D3,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F3" s="12">
+        <f>IF(OR(WEEKDAY(C3)&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C3)=0),IF(E3&gt;0,E3-IF(WEEKDAY(C3)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G3" s="12">
+        <f>IF(OR(WEEKDAY(C3)=1, COUNTIF(Tableau_Pose_Cskn[Date],C3)&gt;0),IF(E3&gt;0,E3-IF(WEEKDAY(C3)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="H3" s="21"/>
+      <c r="M3" s="47">
+        <v>45505</v>
+      </c>
+      <c r="N3" s="52" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>lundi</v>
+      </c>
+      <c r="C4" s="2">
+        <v>45495</v>
+      </c>
+      <c r="D4" s="36">
+        <v>997</v>
+      </c>
+      <c r="E4" s="12">
+        <f>IF(LEN(TRIM(D4))=2,VLOOKUP(TEXT(D4,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D4,1),"0"),POSE_CSKN,3,0))</f>
+        <v>18</v>
+      </c>
+      <c r="F4" s="12">
+        <f>IF(OR(WEEKDAY(C4)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C4)=0),IF(E4&gt;0,E4-IF(WEEKDAY(C4)=7,5,8),0),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G4" s="12">
+        <f>IF(OR(WEEKDAY(C4)=1, COUNTIF(Tableau_Pose_Cskn[Date],C4)&gt;0),IF(E4&gt;0,E4-IF(WEEKDAY(C4)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="21"/>
+      <c r="M4" s="49">
+        <v>45651</v>
+      </c>
+      <c r="N4" s="50" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mardi</v>
+      </c>
+      <c r="C5" s="2">
+        <v>45496</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="12">
+        <f>IF(LEN(TRIM(D5))=2,VLOOKUP(TEXT(D5,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D5,1),"0"),POSE_CSKN,3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="12">
+        <f>IF(OR(WEEKDAY(C5)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C5)=0),IF(E5&gt;0,E5-IF(WEEKDAY(C5)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="12">
+        <f>IF(OR(WEEKDAY(C5)=1, COUNTIF(Tableau_Pose_Cskn[Date],C5)&gt;0),IF(E5&gt;0,E5-IF(WEEKDAY(C5)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="21"/>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mercredi</v>
+      </c>
+      <c r="C6" s="2">
+        <v>45497</v>
+      </c>
+      <c r="D6" s="36">
+        <v>996</v>
+      </c>
+      <c r="E6" s="12">
+        <f>IF(LEN(TRIM(D6))=2,VLOOKUP(TEXT(D6,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D6,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F6" s="12">
+        <f>IF(OR(WEEKDAY(C6)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C6)=0),IF(E6&gt;0,E6-IF(WEEKDAY(C6)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G6" s="12">
+        <f>IF(OR(WEEKDAY(C6)=1, COUNTIF(Tableau_Pose_Cskn[Date],C6)&gt;0),IF(E6&gt;0,E6-IF(WEEKDAY(C6)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="21"/>
+      <c r="K6" s="48">
+        <v>45505</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>jeudi</v>
+      </c>
+      <c r="C7" s="2">
+        <v>45498</v>
+      </c>
+      <c r="D7" s="36">
+        <v>996</v>
+      </c>
+      <c r="E7" s="12">
+        <f>IF(LEN(TRIM(D7))=2,VLOOKUP(TEXT(D7,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D7,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F7" s="12">
+        <f>IF(OR(WEEKDAY(C7)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C7)=0),IF(E7&gt;0,E7-IF(WEEKDAY(C7)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G7" s="12">
+        <f>IF(OR(WEEKDAY(C7)=1, COUNTIF(Tableau_Pose_Cskn[Date],C7)&gt;0),IF(E7&gt;0,E7-IF(WEEKDAY(C7)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="21"/>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>vendredi</v>
+      </c>
+      <c r="C8" s="2">
+        <v>45499</v>
+      </c>
+      <c r="D8" s="36">
+        <v>996</v>
+      </c>
+      <c r="E8" s="12">
+        <f>IF(LEN(TRIM(D8))=2,VLOOKUP(TEXT(D8,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D8,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F8" s="12">
+        <f>IF(OR(WEEKDAY(C8)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C8)=0),IF(E8&gt;0,E8-IF(WEEKDAY(C8)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G8" s="12">
+        <f>IF(OR(WEEKDAY(C8)=1, COUNTIF(Tableau_Pose_Cskn[Date],C8)&gt;0),IF(E8&gt;0,E8-IF(WEEKDAY(C8)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="21"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>samedi</v>
+      </c>
+      <c r="C9" s="2">
+        <v>45500</v>
+      </c>
+      <c r="D9" s="36">
+        <v>996</v>
+      </c>
+      <c r="E9" s="12">
+        <f>IF(LEN(TRIM(D9))=2,VLOOKUP(TEXT(D9,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D9,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F9" s="12">
+        <f>IF(OR(WEEKDAY(C9)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C9)=0),IF(E9&gt;0,E9-IF(WEEKDAY(C9)=7,5,8),0),0)</f>
+        <v>7</v>
+      </c>
+      <c r="G9" s="12">
+        <f>IF(OR(WEEKDAY(C9)=1, COUNTIF(Tableau_Pose_Cskn[Date],C9)&gt;0),IF(E9&gt;0,E9-IF(WEEKDAY(C9)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="21"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B10" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>dimanche</v>
+      </c>
+      <c r="C10" s="2">
+        <v>45501</v>
+      </c>
+      <c r="D10" s="36">
+        <v>996</v>
+      </c>
+      <c r="E10" s="12">
+        <f>IF(LEN(TRIM(D10))=2,VLOOKUP(TEXT(D10,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D10,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F10" s="12">
+        <f>IF(OR(WEEKDAY(C10)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C10)=0),IF(E10&gt;0,E10-IF(WEEKDAY(C10)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G10" s="12">
+        <f>IF(OR(WEEKDAY(C10)=1, COUNTIF(Tableau_Pose_Cskn[Date],C10)&gt;0),IF(E10&gt;0,E10-IF(WEEKDAY(C10)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="H10" s="21"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>lundi</v>
+      </c>
+      <c r="C11" s="2">
+        <v>45502</v>
+      </c>
+      <c r="D11" s="36">
+        <v>997</v>
+      </c>
+      <c r="E11" s="12">
+        <f>IF(LEN(TRIM(D11))=2,VLOOKUP(TEXT(D11,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D11,1),"0"),POSE_CSKN,3,0))</f>
+        <v>18</v>
+      </c>
+      <c r="F11" s="12">
+        <f>IF(OR(WEEKDAY(C11)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C11)=0),IF(E11&gt;0,E11-IF(WEEKDAY(C11)=7,5,8),0),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G11" s="12">
+        <f>IF(OR(WEEKDAY(C11)=1, COUNTIF(Tableau_Pose_Cskn[Date],C11)&gt;0),IF(E11&gt;0,E11-IF(WEEKDAY(C11)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="21"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mardi</v>
+      </c>
+      <c r="C12" s="2">
+        <v>45503</v>
+      </c>
+      <c r="D12" s="36">
+        <v>998</v>
+      </c>
+      <c r="E12" s="12">
+        <f>IF(LEN(TRIM(D12))=2,VLOOKUP(TEXT(D12,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D12,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F12" s="12">
+        <f>IF(OR(WEEKDAY(C12)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C12)=0),IF(E12&gt;0,E12-IF(WEEKDAY(C12)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G12" s="12">
+        <f>IF(OR(WEEKDAY(C12)=1, COUNTIF(Tableau_Pose_Cskn[Date],C12)&gt;0),IF(E12&gt;0,E12-IF(WEEKDAY(C12)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="21"/>
+      <c r="L12" t="b">
+        <f>COUNTIF(Tableau_Pose_Cskn[Date],C14)=0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mercredi</v>
+      </c>
+      <c r="C13" s="2">
+        <v>45504</v>
+      </c>
+      <c r="D13" s="36">
+        <v>998</v>
+      </c>
+      <c r="E13" s="12">
+        <f>IF(LEN(TRIM(D13))=2,VLOOKUP(TEXT(D13,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D13,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F13" s="12">
+        <f>IF(OR(WEEKDAY(C13)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C13)=0),IF(E13&gt;0,E13-IF(WEEKDAY(C13)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G13" s="12">
+        <f>IF(OR(WEEKDAY(C13)=1, COUNTIF(Tableau_Pose_Cskn[Date],C13)&gt;0),IF(E13&gt;0,E13-IF(WEEKDAY(C13)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="21"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>jeudi</v>
+      </c>
+      <c r="C14" s="2">
+        <v>45505</v>
+      </c>
+      <c r="D14" s="36">
+        <v>998</v>
+      </c>
+      <c r="E14" s="12">
+        <f>IF(LEN(TRIM(D14))=2,VLOOKUP(TEXT(D14,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D14,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F14" s="12">
+        <f>IF(OR(WEEKDAY(C14)&lt;&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C14)=0),IF(E14&gt;0,E14-IF(WEEKDAY(C14)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G14" s="12">
+        <f>IF(OR(WEEKDAY(C14)=1, COUNTIF(Tableau_Pose_Cskn[Date],C14)&gt;0),IF(E14&gt;0,E14-IF(WEEKDAY(C14)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="H14" s="21"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>vendredi</v>
+      </c>
+      <c r="C15" s="2">
+        <v>45506</v>
+      </c>
+      <c r="D15" s="36">
+        <v>998</v>
+      </c>
+      <c r="E15" s="12">
+        <f>IF(LEN(TRIM(D15))=2,VLOOKUP(TEXT(D15,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D15,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F15" s="12">
+        <f>IF(WEEKDAY(C15)&lt;&gt;1,IF(E15&gt;0,E15-IF(WEEKDAY(C15)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G15" s="12">
+        <f>IF(OR(WEEKDAY(C15)=1, COUNTIF(Tableau_Pose_Cskn[Date],C15)&gt;0),IF(E15&gt;0,E15-IF(WEEKDAY(C15)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="21"/>
+      <c r="L15" t="b">
+        <f>OR(WEEKDAY(C3)&gt;1, COUNTIF(Tableau_Pose_Cskn[Date],C3)=0)</f>
+        <v>1</v>
+      </c>
+      <c r="N15" t="b">
+        <f>COUNTIF(Tableau_Pose_Cskn[Date],C3)=0</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>samedi</v>
+      </c>
+      <c r="C16" s="2">
+        <v>45507</v>
+      </c>
+      <c r="D16" s="36">
+        <v>998</v>
+      </c>
+      <c r="E16" s="12">
+        <f>IF(LEN(TRIM(D16))=2,VLOOKUP(TEXT(D16,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D16,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F16" s="12">
+        <f>IF(WEEKDAY(C16)&lt;&gt;1,IF(E16&gt;0,E16-IF(WEEKDAY(C16)=7,5,8),0),0)</f>
+        <v>7</v>
+      </c>
+      <c r="G16" s="12">
+        <f>IF(OR(WEEKDAY(C16)=1, COUNTIF(Tableau_Pose_Cskn[Date],C16)&gt;0),IF(E16&gt;0,E16-IF(WEEKDAY(C16)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="21"/>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B17" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>dimanche</v>
+      </c>
+      <c r="C17" s="2">
+        <v>45508</v>
+      </c>
+      <c r="D17" s="36">
+        <v>998</v>
+      </c>
+      <c r="E17" s="12">
+        <f>IF(LEN(TRIM(D17))=2,VLOOKUP(TEXT(D17,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D17,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F17" s="12">
+        <f>IF(WEEKDAY(C17)&lt;&gt;1,IF(E17&gt;0,E17-IF(WEEKDAY(C17)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="12">
+        <f>IF(OR(WEEKDAY(C17)=1, COUNTIF(Tableau_Pose_Cskn[Date],C17)&gt;0),IF(E17&gt;0,E17-IF(WEEKDAY(C17)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="H17" s="21"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>lundi</v>
+      </c>
+      <c r="C18" s="2">
+        <v>45509</v>
+      </c>
+      <c r="D18" s="36">
+        <v>997</v>
+      </c>
+      <c r="E18" s="12">
+        <f>IF(LEN(TRIM(D18))=2,VLOOKUP(TEXT(D18,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D18,1),"0"),POSE_CSKN,3,0))</f>
+        <v>18</v>
+      </c>
+      <c r="F18" s="12">
+        <f>IF(WEEKDAY(C18)&lt;&gt;1,IF(E18&gt;0,E18-IF(WEEKDAY(C18)=7,5,8),0),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G18" s="12">
+        <f>IF(OR(WEEKDAY(C18)=1, COUNTIF(Tableau_Pose_Cskn[Date],C18)&gt;0),IF(E18&gt;0,E18-IF(WEEKDAY(C18)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="21"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mardi</v>
+      </c>
+      <c r="C19" s="2">
+        <v>45510</v>
+      </c>
+      <c r="D19" s="36">
+        <v>12</v>
+      </c>
+      <c r="E19" s="12">
+        <f>IF(LEN(TRIM(D19))=2,VLOOKUP(TEXT(D19,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D19,1),"0"),POSE_CSKN,3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="12">
+        <f>IF(WEEKDAY(C19)&lt;&gt;1,IF(E19&gt;0,E19-IF(WEEKDAY(C19)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="12">
+        <f>IF(OR(WEEKDAY(C19)=1, COUNTIF(Tableau_Pose_Cskn[Date],C19)&gt;0),IF(E19&gt;0,E19-IF(WEEKDAY(C19)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="21"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mercredi</v>
+      </c>
+      <c r="C20" s="2">
+        <v>45511</v>
+      </c>
+      <c r="D20" s="36">
+        <v>996</v>
+      </c>
+      <c r="E20" s="12">
+        <f>IF(LEN(TRIM(D20))=2,VLOOKUP(TEXT(D20,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D20,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F20" s="12">
+        <f>IF(WEEKDAY(C20)&lt;&gt;1,IF(E20&gt;0,E20-IF(WEEKDAY(C20)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G20" s="12">
+        <f>IF(OR(WEEKDAY(C20)=1, COUNTIF(Tableau_Pose_Cskn[Date],C20)&gt;0),IF(E20&gt;0,E20-IF(WEEKDAY(C20)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="21"/>
+      <c r="K20" s="28">
+        <v>1.3</v>
+      </c>
+      <c r="L20" s="28">
+        <v>1.6</v>
+      </c>
+      <c r="M20" s="28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>jeudi</v>
+      </c>
+      <c r="C21" s="2">
+        <v>45512</v>
+      </c>
+      <c r="D21" s="36">
+        <v>996</v>
+      </c>
+      <c r="E21" s="12">
+        <f>IF(LEN(TRIM(D21))=2,VLOOKUP(TEXT(D21,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D21,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F21" s="12">
+        <f>IF(WEEKDAY(C21)&lt;&gt;1,IF(E21&gt;0,E21-IF(WEEKDAY(C21)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G21" s="12">
+        <f>IF(OR(WEEKDAY(C21)=1, COUNTIF(Tableau_Pose_Cskn[Date],C21)&gt;0),IF(E21&gt;0,E21-IF(WEEKDAY(C21)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="21"/>
+      <c r="J21" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="K21" s="12">
+        <v>6</v>
+      </c>
+      <c r="L21" s="12">
+        <v>15</v>
+      </c>
+      <c r="M21" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>vendredi</v>
+      </c>
+      <c r="C22" s="2">
+        <v>45513</v>
+      </c>
+      <c r="D22" s="36">
+        <v>996</v>
+      </c>
+      <c r="E22" s="12">
+        <f>IF(LEN(TRIM(D22))=2,VLOOKUP(TEXT(D22,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D22,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F22" s="12">
+        <f>IF(WEEKDAY(C22)&lt;&gt;1,IF(E22&gt;0,E22-IF(WEEKDAY(C22)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G22" s="12">
+        <f>IF(OR(WEEKDAY(C22)=1, COUNTIF(Tableau_Pose_Cskn[Date],C22)&gt;0),IF(E22&gt;0,E22-IF(WEEKDAY(C22)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="21"/>
+      <c r="J22" s="27" t="s">
+        <v>261</v>
+      </c>
+      <c r="K22" s="12">
+        <v>6</v>
+      </c>
+      <c r="L22" s="12">
+        <v>27</v>
+      </c>
+      <c r="M22" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>samedi</v>
+      </c>
+      <c r="C23" s="2">
+        <v>45514</v>
+      </c>
+      <c r="D23" s="36">
+        <v>996</v>
+      </c>
+      <c r="E23" s="12">
+        <f>IF(LEN(TRIM(D23))=2,VLOOKUP(TEXT(D23,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D23,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F23" s="12">
+        <f>IF(WEEKDAY(C23)&lt;&gt;1,IF(E23&gt;0,E23-IF(WEEKDAY(C23)=7,5,8),0),0)</f>
+        <v>7</v>
+      </c>
+      <c r="G23" s="12">
+        <f>IF(OR(WEEKDAY(C23)=1, COUNTIF(Tableau_Pose_Cskn[Date],C23)&gt;0),IF(E23&gt;0,E23-IF(WEEKDAY(C23)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="21"/>
+      <c r="J23" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="K23" s="12">
+        <v>6</v>
+      </c>
+      <c r="L23" s="29">
+        <v>15</v>
+      </c>
+      <c r="M23" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B24" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>dimanche</v>
+      </c>
+      <c r="C24" s="2">
+        <v>45515</v>
+      </c>
+      <c r="D24" s="36">
+        <v>996</v>
+      </c>
+      <c r="E24" s="12">
+        <f>IF(LEN(TRIM(D24))=2,VLOOKUP(TEXT(D24,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D24,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F24" s="12">
+        <f>IF(WEEKDAY(C24)&lt;&gt;1,IF(E24&gt;0,E24-IF(WEEKDAY(C24)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="12">
+        <f>IF(OR(WEEKDAY(C24)=1, COUNTIF(Tableau_Pose_Cskn[Date],C24)&gt;0),IF(E24&gt;0,E24-IF(WEEKDAY(C24)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="H24" s="21"/>
+      <c r="J24" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="K24" s="12">
+        <v>6</v>
+      </c>
+      <c r="L24" s="29">
+        <v>15</v>
+      </c>
+      <c r="M24" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>lundi</v>
+      </c>
+      <c r="C25" s="2">
+        <v>45516</v>
+      </c>
+      <c r="D25" s="36">
+        <v>997</v>
+      </c>
+      <c r="E25" s="12">
+        <f>IF(LEN(TRIM(D25))=2,VLOOKUP(TEXT(D25,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D25,1),"0"),POSE_CSKN,3,0))</f>
+        <v>18</v>
+      </c>
+      <c r="F25" s="12">
+        <f>IF(WEEKDAY(C25)&lt;&gt;1,IF(E25&gt;0,E25-IF(WEEKDAY(C25)=7,5,8),0),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G25" s="12">
+        <f>IF(OR(WEEKDAY(C25)=1, COUNTIF(Tableau_Pose_Cskn[Date],C25)&gt;0),IF(E25&gt;0,E25-IF(WEEKDAY(C25)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="21"/>
+      <c r="J25" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="K25" s="12">
+        <v>6</v>
+      </c>
+      <c r="L25" s="29">
+        <v>4</v>
+      </c>
+      <c r="M25" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" ht="13" x14ac:dyDescent="0.3">
+      <c r="B26" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mardi</v>
+      </c>
+      <c r="C26" s="2">
+        <v>45517</v>
+      </c>
+      <c r="D26" s="36">
+        <v>998</v>
+      </c>
+      <c r="E26" s="12">
+        <f>IF(LEN(TRIM(D26))=2,VLOOKUP(TEXT(D26,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D26,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F26" s="12">
+        <f>IF(WEEKDAY(C26)&lt;&gt;1,IF(E26&gt;0,E26-IF(WEEKDAY(C26)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G26" s="12">
+        <f>IF(OR(WEEKDAY(C26)=1, COUNTIF(Tableau_Pose_Cskn[Date],C26)&gt;0),IF(E26&gt;0,E26-IF(WEEKDAY(C26)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="21"/>
+      <c r="J26" s="44" t="s">
+        <v>288</v>
+      </c>
+      <c r="K26" s="12">
+        <v>0</v>
+      </c>
+      <c r="L26" s="29">
+        <v>0</v>
+      </c>
+      <c r="M26" s="12">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mercredi</v>
+      </c>
+      <c r="C27" s="2">
+        <v>45518</v>
+      </c>
+      <c r="D27" s="36">
+        <v>998</v>
+      </c>
+      <c r="E27" s="12">
+        <f>IF(LEN(TRIM(D27))=2,VLOOKUP(TEXT(D27,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D27,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F27" s="12">
+        <f>IF(WEEKDAY(C27)&lt;&gt;1,IF(E27&gt;0,E27-IF(WEEKDAY(C27)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G27" s="12">
+        <f>IF(OR(WEEKDAY(C27)=1, COUNTIF(Tableau_Pose_Cskn[Date],C27)&gt;0),IF(E27&gt;0,E27-IF(WEEKDAY(C27)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="21"/>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>jeudi</v>
+      </c>
+      <c r="C28" s="2">
+        <v>45519</v>
+      </c>
+      <c r="D28" s="36">
+        <v>998</v>
+      </c>
+      <c r="E28" s="12">
+        <f>IF(LEN(TRIM(D28))=2,VLOOKUP(TEXT(D28,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D28,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F28" s="12">
+        <f>IF(WEEKDAY(C28)&lt;&gt;1,IF(E28&gt;0,E28-IF(WEEKDAY(C28)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G28" s="12">
+        <f>IF(OR(WEEKDAY(C28)=1, COUNTIF(Tableau_Pose_Cskn[Date],C28)&gt;0),IF(E28&gt;0,E28-IF(WEEKDAY(C28)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="21"/>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>vendredi</v>
+      </c>
+      <c r="C29" s="2">
+        <v>45520</v>
+      </c>
+      <c r="D29" s="36">
+        <v>998</v>
+      </c>
+      <c r="E29" s="12">
+        <f>IF(LEN(TRIM(D29))=2,VLOOKUP(TEXT(D29,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D29,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F29" s="12">
+        <f>IF(WEEKDAY(C29)&lt;&gt;1,IF(E29&gt;0,E29-IF(WEEKDAY(C29)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="G29" s="12">
+        <f>IF(OR(WEEKDAY(C29)=1, COUNTIF(Tableau_Pose_Cskn[Date],C29)&gt;0),IF(E29&gt;0,E29-IF(WEEKDAY(C29)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="21"/>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>samedi</v>
+      </c>
+      <c r="C30" s="2">
+        <v>45521</v>
+      </c>
+      <c r="D30" s="36">
+        <v>12</v>
+      </c>
+      <c r="E30" s="12">
+        <f>IF(LEN(TRIM(D30))=2,VLOOKUP(TEXT(D30,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D30,1),"0"),POSE_CSKN,3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="12">
+        <f>IF(WEEKDAY(C30)&lt;&gt;1,IF(E30&gt;0,E30-IF(WEEKDAY(C30)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="12">
+        <f>IF(OR(WEEKDAY(C30)=1, COUNTIF(Tableau_Pose_Cskn[Date],C30)&gt;0),IF(E30&gt;0,E30-IF(WEEKDAY(C30)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="21"/>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B31" s="23" t="str">
+        <f t="shared" si="0"/>
+        <v>dimanche</v>
+      </c>
+      <c r="C31" s="2">
+        <v>45522</v>
+      </c>
+      <c r="D31" s="36">
+        <v>998</v>
+      </c>
+      <c r="E31" s="12">
+        <f>IF(LEN(TRIM(D31))=2,VLOOKUP(TEXT(D31,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D31,1),"0"),POSE_CSKN,3,0))</f>
+        <v>12</v>
+      </c>
+      <c r="F31" s="12">
+        <f>IF(WEEKDAY(C31)&lt;&gt;1,IF(E31&gt;0,E31-IF(WEEKDAY(C31)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="12">
+        <f>IF(OR(WEEKDAY(C31)=1, COUNTIF(Tableau_Pose_Cskn[Date],C31)&gt;0),IF(E31&gt;0,E31-IF(WEEKDAY(C31)=7,5,8),0),0)</f>
+        <v>4</v>
+      </c>
+      <c r="H31" s="21"/>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>lundi</v>
+      </c>
+      <c r="C32" s="2">
+        <v>45523</v>
+      </c>
+      <c r="D32" s="36">
+        <v>997</v>
+      </c>
+      <c r="E32" s="12">
+        <f>IF(LEN(TRIM(D32))=2,VLOOKUP(TEXT(D32,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D32,1),"0"),POSE_CSKN,3,0))</f>
+        <v>18</v>
+      </c>
+      <c r="F32" s="12">
+        <f>IF(WEEKDAY(C32)&lt;&gt;1,IF(E32&gt;0,E32-IF(WEEKDAY(C32)=7,5,8),0),0)</f>
+        <v>10</v>
+      </c>
+      <c r="G32" s="12">
+        <f>IF(OR(WEEKDAY(C32)=1, COUNTIF(Tableau_Pose_Cskn[Date],C32)&gt;0),IF(E32&gt;0,E32-IF(WEEKDAY(C32)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="21"/>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>mardi</v>
+      </c>
+      <c r="C33" s="2">
+        <v>45524</v>
+      </c>
+      <c r="D33" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="12">
+        <f>IF(LEN(TRIM(D33))=2,VLOOKUP(TEXT(D33,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D33,1),"0"),POSE_CSKN,3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="12">
+        <f>IF(WEEKDAY(C33)&lt;&gt;1,IF(E33&gt;0,E33-IF(WEEKDAY(C33)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="12">
+        <f>IF(OR(WEEKDAY(C33)=1, COUNTIF(Tableau_Pose_Cskn[Date],C33)&gt;0),IF(E33&gt;0,E33-IF(WEEKDAY(C33)=7,5,8),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="21"/>
+    </row>
+    <row r="34" spans="2:8" ht="13" x14ac:dyDescent="0.3">
+      <c r="E34" s="40">
+        <f t="shared" ref="E34:G34" si="1">SUM(E3:E33)</f>
+        <v>354</v>
+      </c>
+      <c r="F34" s="40">
+        <f t="shared" si="1"/>
+        <v>135</v>
+      </c>
+      <c r="G34" s="40">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5287AAF-25F6-426B-93DC-326260F9D879}">
+  <dimension ref="B3:M100"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="31.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:13" ht="13" x14ac:dyDescent="0.3">
+      <c r="C3" s="35" t="s">
+        <v>286</v>
+      </c>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="K3" s="35" t="s">
+        <v>287</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+    </row>
+    <row r="5" spans="2:13" ht="26" x14ac:dyDescent="0.25">
+      <c r="B5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>282</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="M5" s="34" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E6" s="10">
+        <v>5</v>
+      </c>
+      <c r="F6" s="12">
+        <v>0</v>
+      </c>
+      <c r="G6" s="12">
+        <v>0</v>
+      </c>
+      <c r="K6" s="14">
+        <v>0</v>
+      </c>
+      <c r="L6" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="M6" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E7" s="10">
+        <v>0</v>
+      </c>
+      <c r="F7" s="12">
+        <v>0</v>
+      </c>
+      <c r="G7" s="12">
+        <v>0</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="M7" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E8" s="10">
+        <v>8</v>
+      </c>
+      <c r="F8" s="12">
+        <v>0</v>
+      </c>
+      <c r="G8" s="12">
+        <v>0</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="M8" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E9" s="10">
+        <v>0</v>
+      </c>
+      <c r="F9" s="12">
+        <v>0</v>
+      </c>
+      <c r="G9" s="12">
+        <v>0</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="M9" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E10" s="10">
+        <v>11</v>
+      </c>
+      <c r="F10" s="12">
+        <v>0</v>
+      </c>
+      <c r="G10" s="12">
+        <v>0</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="M10" s="12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E11" s="10">
+        <v>15</v>
+      </c>
+      <c r="F11" s="12">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <v>0</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="M11" s="12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0</v>
+      </c>
+      <c r="F12" s="12">
+        <v>0</v>
+      </c>
+      <c r="G12" s="12">
+        <v>0</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="M12" s="12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E13" s="10">
+        <v>0</v>
+      </c>
+      <c r="F13" s="12">
+        <v>0</v>
+      </c>
+      <c r="G13" s="12">
+        <v>0</v>
+      </c>
+      <c r="K13" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="M13" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E14" s="10">
+        <v>8</v>
+      </c>
+      <c r="F14" s="12">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E15" s="10">
+        <v>0</v>
+      </c>
+      <c r="F15" s="12">
+        <v>0</v>
+      </c>
+      <c r="G15" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E16" s="10">
+        <v>6</v>
+      </c>
+      <c r="F16" s="12">
+        <v>0</v>
+      </c>
+      <c r="G16" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E17" s="10">
+        <v>0</v>
+      </c>
+      <c r="F17" s="12">
+        <v>0</v>
+      </c>
+      <c r="G17" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E18" s="10">
+        <v>45</v>
+      </c>
+      <c r="F18" s="12">
+        <v>0</v>
+      </c>
+      <c r="G18" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E19" s="10">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12">
+        <v>0</v>
+      </c>
+      <c r="G19" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E20" s="10">
+        <v>0</v>
+      </c>
+      <c r="F20" s="12">
+        <v>0</v>
+      </c>
+      <c r="G20" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E21" s="10">
+        <v>1</v>
+      </c>
+      <c r="F21" s="12">
+        <v>1</v>
+      </c>
+      <c r="G21" s="12"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E22" s="10">
+        <v>1</v>
+      </c>
+      <c r="F22" s="12">
+        <v>1</v>
+      </c>
+      <c r="G22" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E23" s="10">
+        <v>1</v>
+      </c>
+      <c r="F23" s="12">
+        <v>1</v>
+      </c>
+      <c r="G23" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E24" s="10">
+        <v>1</v>
+      </c>
+      <c r="F24" s="12">
+        <v>1</v>
+      </c>
+      <c r="G24" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E25" s="10">
+        <v>0</v>
+      </c>
+      <c r="F25" s="12">
+        <v>1</v>
+      </c>
+      <c r="G25" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E26" s="10">
+        <v>1</v>
+      </c>
+      <c r="F26" s="12">
+        <v>1</v>
+      </c>
+      <c r="G26" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E27" s="10">
+        <v>0</v>
+      </c>
+      <c r="F27" s="12">
+        <v>1</v>
+      </c>
+      <c r="G27" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E28" s="10">
+        <v>1</v>
+      </c>
+      <c r="F28" s="12">
+        <v>1</v>
+      </c>
+      <c r="G28" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E29" s="10">
+        <v>1</v>
+      </c>
+      <c r="F29" s="12">
+        <v>1</v>
+      </c>
+      <c r="G29" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E30" s="10">
+        <v>1</v>
+      </c>
+      <c r="F30" s="12">
+        <v>1</v>
+      </c>
+      <c r="G30" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E31" s="10">
+        <v>0</v>
+      </c>
+      <c r="F31" s="12">
+        <v>1</v>
+      </c>
+      <c r="G31" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E32" s="10">
+        <v>0</v>
+      </c>
+      <c r="F32" s="12">
+        <v>1</v>
+      </c>
+      <c r="G32" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E33" s="10">
+        <v>0</v>
+      </c>
+      <c r="F33" s="12">
+        <v>1</v>
+      </c>
+      <c r="G33" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E34" s="10">
+        <v>0</v>
+      </c>
+      <c r="F34" s="12">
+        <v>1</v>
+      </c>
+      <c r="G34" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E35" s="10">
+        <v>0</v>
+      </c>
+      <c r="F35" s="12">
+        <v>1</v>
+      </c>
+      <c r="G35" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E36" s="10">
+        <v>0</v>
+      </c>
+      <c r="F36" s="12">
+        <v>1</v>
+      </c>
+      <c r="G36" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E37" s="10">
+        <v>0</v>
+      </c>
+      <c r="F37" s="12">
+        <v>1</v>
+      </c>
+      <c r="G37" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E38" s="10">
+        <v>0</v>
+      </c>
+      <c r="F38" s="12">
+        <v>1</v>
+      </c>
+      <c r="G38" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E39" s="10">
+        <v>0</v>
+      </c>
+      <c r="F39" s="12">
+        <v>1</v>
+      </c>
+      <c r="G39" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E40" s="10">
+        <v>0</v>
+      </c>
+      <c r="F40" s="12">
+        <v>1</v>
+      </c>
+      <c r="G40" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E41" s="10">
+        <v>0</v>
+      </c>
+      <c r="F41" s="12">
+        <v>1</v>
+      </c>
+      <c r="G41" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E42" s="10">
+        <v>0</v>
+      </c>
+      <c r="F42" s="12">
+        <v>1</v>
+      </c>
+      <c r="G42" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E43" s="10">
+        <v>0</v>
+      </c>
+      <c r="F43" s="12">
+        <v>1</v>
+      </c>
+      <c r="G43" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E44" s="10">
+        <v>0</v>
+      </c>
+      <c r="F44" s="12">
+        <v>1</v>
+      </c>
+      <c r="G44" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" ht="25" x14ac:dyDescent="0.25">
+      <c r="B45" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E45" s="10">
+        <v>0</v>
+      </c>
+      <c r="F45" s="12">
+        <v>1</v>
+      </c>
+      <c r="G45" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B46" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E46" s="10">
+        <v>0</v>
+      </c>
+      <c r="F46" s="12">
+        <v>1</v>
+      </c>
+      <c r="G46" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B47" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E47" s="10">
+        <v>0</v>
+      </c>
+      <c r="F47" s="12">
+        <v>1</v>
+      </c>
+      <c r="G47" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B48" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E48" s="10">
+        <v>0</v>
+      </c>
+      <c r="F48" s="12">
+        <v>1</v>
+      </c>
+      <c r="G48" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E49" s="10">
+        <v>0</v>
+      </c>
+      <c r="F49" s="12">
+        <v>1</v>
+      </c>
+      <c r="G49" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E50" s="10">
+        <v>1</v>
+      </c>
+      <c r="F50" s="12">
+        <v>1</v>
+      </c>
+      <c r="G50" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B51" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E51" s="10">
+        <v>1</v>
+      </c>
+      <c r="F51" s="12">
+        <v>1</v>
+      </c>
+      <c r="G51" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E52" s="10">
+        <v>1</v>
+      </c>
+      <c r="F52" s="12">
+        <v>1</v>
+      </c>
+      <c r="G52" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E53" s="10">
+        <v>0</v>
+      </c>
+      <c r="F53" s="12">
+        <v>1</v>
+      </c>
+      <c r="G53" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E54" s="10">
+        <v>1</v>
+      </c>
+      <c r="F54" s="12">
+        <v>1</v>
+      </c>
+      <c r="G54" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B55" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E55" s="10">
+        <v>1</v>
+      </c>
+      <c r="F55" s="12">
+        <v>1</v>
+      </c>
+      <c r="G55" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E56" s="10">
+        <v>0</v>
+      </c>
+      <c r="F56" s="12">
+        <v>1</v>
+      </c>
+      <c r="G56" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B57" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E57" s="10">
+        <v>0</v>
+      </c>
+      <c r="F57" s="12">
+        <v>1</v>
+      </c>
+      <c r="G57" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B58" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E58" s="10">
+        <v>0</v>
+      </c>
+      <c r="F58" s="12">
+        <v>1</v>
+      </c>
+      <c r="G58" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B59" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E59" s="10">
+        <v>1</v>
+      </c>
+      <c r="F59" s="12">
+        <v>1</v>
+      </c>
+      <c r="G59" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B60" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E60" s="10">
+        <v>1</v>
+      </c>
+      <c r="F60" s="12">
+        <v>1</v>
+      </c>
+      <c r="G60" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B61" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E61" s="10">
+        <v>1</v>
+      </c>
+      <c r="F61" s="12">
+        <v>1</v>
+      </c>
+      <c r="G61" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B62" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E62" s="10">
+        <v>1</v>
+      </c>
+      <c r="F62" s="12">
+        <v>1</v>
+      </c>
+      <c r="G62" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B63" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E63" s="10">
+        <v>1</v>
+      </c>
+      <c r="F63" s="12">
+        <v>1</v>
+      </c>
+      <c r="G63" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B64" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E64" s="10">
+        <v>0</v>
+      </c>
+      <c r="F64" s="12">
+        <v>1</v>
+      </c>
+      <c r="G64" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B65" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E65" s="10">
+        <v>0</v>
+      </c>
+      <c r="F65" s="12">
+        <v>1</v>
+      </c>
+      <c r="G65" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B66" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E66" s="10">
+        <v>0</v>
+      </c>
+      <c r="F66" s="12">
+        <v>1</v>
+      </c>
+      <c r="G66" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B67" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E67" s="10">
+        <v>1</v>
+      </c>
+      <c r="F67" s="12">
+        <v>1</v>
+      </c>
+      <c r="G67" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B68" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E68" s="10">
+        <v>1</v>
+      </c>
+      <c r="F68" s="12">
+        <v>1</v>
+      </c>
+      <c r="G68" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B69" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E69" s="10">
+        <v>0</v>
+      </c>
+      <c r="F69" s="12">
+        <v>1</v>
+      </c>
+      <c r="G69" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B70" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E70" s="10">
+        <v>0</v>
+      </c>
+      <c r="F70" s="12">
+        <v>1</v>
+      </c>
+      <c r="G70" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B71" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E71" s="10">
+        <v>0</v>
+      </c>
+      <c r="F71" s="12">
+        <v>1</v>
+      </c>
+      <c r="G71" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E72" s="10">
+        <v>0</v>
+      </c>
+      <c r="F72" s="12">
+        <v>1</v>
+      </c>
+      <c r="G72" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B73" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E73" s="10">
+        <v>0</v>
+      </c>
+      <c r="F73" s="12">
+        <v>1</v>
+      </c>
+      <c r="G73" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B74" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E74" s="10">
+        <v>0</v>
+      </c>
+      <c r="F74" s="12">
+        <v>1</v>
+      </c>
+      <c r="G74" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B75" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E75" s="10">
+        <v>0</v>
+      </c>
+      <c r="F75" s="12">
+        <v>1</v>
+      </c>
+      <c r="G75" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B76" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E76" s="10">
+        <v>1</v>
+      </c>
+      <c r="F76" s="12">
+        <v>1</v>
+      </c>
+      <c r="G76" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B77" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E77" s="10">
+        <v>0</v>
+      </c>
+      <c r="F77" s="12">
+        <v>1</v>
+      </c>
+      <c r="G77" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B78" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E78" s="10">
+        <v>1</v>
+      </c>
+      <c r="F78" s="12">
+        <v>1</v>
+      </c>
+      <c r="G78" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B79" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E79" s="10">
+        <v>0</v>
+      </c>
+      <c r="F79" s="12">
+        <v>1</v>
+      </c>
+      <c r="G79" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B80" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E80" s="10">
+        <v>0</v>
+      </c>
+      <c r="F80" s="12">
+        <v>1</v>
+      </c>
+      <c r="G80" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B81" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E81" s="10">
+        <v>0</v>
+      </c>
+      <c r="F81" s="12">
+        <v>1</v>
+      </c>
+      <c r="G81" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B82" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E82" s="10">
+        <v>0</v>
+      </c>
+      <c r="F82" s="12">
+        <v>1</v>
+      </c>
+      <c r="G82" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B83" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E83" s="10">
+        <v>0</v>
+      </c>
+      <c r="F83" s="12">
+        <v>1</v>
+      </c>
+      <c r="G83" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B84" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E84" s="10">
+        <v>0</v>
+      </c>
+      <c r="F84" s="12">
+        <v>1</v>
+      </c>
+      <c r="G84" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B85" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E85" s="10">
+        <v>0</v>
+      </c>
+      <c r="F85" s="12">
+        <v>1</v>
+      </c>
+      <c r="G85" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B86" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E86" s="10">
+        <v>0</v>
+      </c>
+      <c r="F86" s="12">
+        <v>1</v>
+      </c>
+      <c r="G86" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B87" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E87" s="10">
+        <v>0</v>
+      </c>
+      <c r="F87" s="12">
+        <v>1</v>
+      </c>
+      <c r="G87" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B88" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E88" s="10">
+        <v>0</v>
+      </c>
+      <c r="F88" s="12">
+        <v>1</v>
+      </c>
+      <c r="G88" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B89" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E89" s="10">
+        <v>0</v>
+      </c>
+      <c r="F89" s="12">
+        <v>1</v>
+      </c>
+      <c r="G89" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B90" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E90" s="10">
+        <v>0</v>
+      </c>
+      <c r="F90" s="12">
+        <v>1</v>
+      </c>
+      <c r="G90" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B91" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E91" s="10">
+        <v>0</v>
+      </c>
+      <c r="F91" s="12">
+        <v>1</v>
+      </c>
+      <c r="G91" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B92" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E92" s="10">
+        <v>0</v>
+      </c>
+      <c r="F92" s="12">
+        <v>1</v>
+      </c>
+      <c r="G92" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B93" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E93" s="10">
+        <v>0</v>
+      </c>
+      <c r="F93" s="12">
+        <v>1</v>
+      </c>
+      <c r="G93" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B94" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E94" s="10">
+        <v>0</v>
+      </c>
+      <c r="F94" s="12">
+        <v>1</v>
+      </c>
+      <c r="G94" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="95" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B95" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E95" s="10">
+        <v>0</v>
+      </c>
+      <c r="F95" s="12">
+        <v>1</v>
+      </c>
+      <c r="G95" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B96" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E96" s="10">
+        <v>0</v>
+      </c>
+      <c r="F96" s="12">
+        <v>1</v>
+      </c>
+      <c r="G96" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B97" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E97" s="10">
+        <v>0</v>
+      </c>
+      <c r="F97" s="12">
+        <v>1</v>
+      </c>
+      <c r="G97" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B98" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E98" s="10">
+        <v>0</v>
+      </c>
+      <c r="F98" s="12">
+        <v>1</v>
+      </c>
+      <c r="G98" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B99" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E99" s="10">
+        <v>0</v>
+      </c>
+      <c r="F99" s="12">
+        <v>1</v>
+      </c>
+      <c r="G99" s="12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B100" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="E100" s="10">
+        <v>0</v>
+      </c>
+      <c r="F100" s="12">
+        <v>1</v>
+      </c>
+      <c r="G100" s="12">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="K3:M3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mise à jour du 01 oct 2026
</commit_message>
<xml_diff>
--- a/POINTAGE_BRUT_AOUT_24.xlsx
+++ b/POINTAGE_BRUT_AOUT_24.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B.NIMI\Desktop\DIVERS\Fichiers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C4CA8E6-F310-4930-B0B2-34E4B4523B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9394A5AD-477A-4D35-815C-24AA611258C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="POINTAGES" sheetId="1" r:id="rId1"/>
     <sheet name="HS" sheetId="3" r:id="rId2"/>
-    <sheet name="Feuil1" sheetId="4" r:id="rId3"/>
+    <sheet name="A_SUPPRIMER" sheetId="4" r:id="rId3"/>
     <sheet name="Feuil2" sheetId="5" r:id="rId4"/>
-    <sheet name="A_SUPPRIMER_APRES" sheetId="7" r:id="rId5"/>
-    <sheet name="Configurations" sheetId="6" r:id="rId6"/>
+    <sheet name="PROPOS_GPT" sheetId="8" r:id="rId5"/>
+    <sheet name="A_SUPPRIMER_APRES" sheetId="7" r:id="rId6"/>
+    <sheet name="Configurations" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Feuil1!$C$4:$K$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">A_SUPPRIMER!$C$4:$K$35</definedName>
     <definedName name="POSE_CSKN">Configurations!$K$5:$M$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="314">
   <si>
     <t>Matricule</t>
   </si>
@@ -972,6 +973,18 @@
   </si>
   <si>
     <t>Je souhaite que tu m'aide avec des formules Excel pour reproduire le tableau ci-dessous :</t>
+  </si>
+  <si>
+    <t>HS 130%</t>
+  </si>
+  <si>
+    <t>HS 160%</t>
+  </si>
+  <si>
+    <t>HS 200%</t>
+  </si>
+  <si>
+    <t>Debut semaine</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1037,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1049,8 +1062,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1130,11 +1149,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1219,17 +1277,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1246,14 +1298,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1265,11 +1311,358 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="22">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1404,14 +1797,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38945EDF-6FD5-4996-A655-EE0F60A9CF58}" name="Tableau_Pose_Cskn" displayName="Tableau_Pose_Cskn" ref="N2:O4" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38945EDF-6FD5-4996-A655-EE0F60A9CF58}" name="Tableau_Pose_Cskn" displayName="Tableau_Pose_Cskn" ref="N2:O4" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19" totalsRowBorderDxfId="18">
   <autoFilter ref="N2:O4" xr:uid="{38945EDF-6FD5-4996-A655-EE0F60A9CF58}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{FA25F88B-AD6F-4A5D-8F20-994C35E94325}" name="Date" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{BF59DA52-CD1D-4A0A-887A-22E32213672D}" name="Jour" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{FA25F88B-AD6F-4A5D-8F20-994C35E94325}" name="Date" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{BF59DA52-CD1D-4A0A-887A-22E32213672D}" name="Jour" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{73A250A8-CDF1-4A04-886C-8F7DE0BF6CFE}" name="TB_Prestattion" displayName="TB_Prestattion" ref="C2:H33" totalsRowShown="0" headerRowBorderDxfId="6" tableBorderDxfId="7">
+  <autoFilter ref="C2:H33" xr:uid="{73A250A8-CDF1-4A04-886C-8F7DE0BF6CFE}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{31C8EF65-8210-418D-BED8-5C1AB1591069}" name="Date" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{C2559552-F5D1-4E81-97F4-C6749B3A3327}" name="Pose" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{AB6DAB21-43D1-4DAB-9C45-7AA38C41184A}" name="Heures Légales" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{4FA4F01A-4FEB-4577-B5FC-3A64DFEC109D}" name="Prestation totale" dataDxfId="2">
+      <calculatedColumnFormula>IF(LEN(TRIM(D3))=2,VLOOKUP(TEXT(D3,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D3,1),"0"),POSE_CSKN,3,0))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{A61CA07E-E25C-4A5C-BE40-B7CAC4FC7DA8}" name="HS Jr  ouvré" dataDxfId="1">
+      <calculatedColumnFormula>IF(AND(WEEKDAY(C3)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C3)=0),IF(F3&gt;0,F3-IF(WEEKDAY(C3)=7,5,8),0),0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{943B10D3-AF02-4B96-9B81-D267D9EFC397}" name="HS Jr non ouvré" dataDxfId="0">
+      <calculatedColumnFormula>IF(OR(WEEKDAY(C3)=1,COUNTIF(Tableau_Pose_Cskn[Date],C3)&gt;0),IF(F3&gt;0,F3-IF(WEEKDAY(C3)=7,5,8),0),0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BC97A63C-6FDD-44E7-BB1C-27BFBB31C8AF}" name="Tableau_Prestation" displayName="Tableau_Prestation" ref="A1:D32" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13">
+  <autoFilter ref="A1:D32" xr:uid="{BC97A63C-6FDD-44E7-BB1C-27BFBB31C8AF}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{5A3D78EF-7B5D-458C-A425-A90104C175DC}" name="Jour" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{876114C1-D4B8-40B3-B6D9-91F7865B2D14}" name="Date" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{4C2937B3-84AA-4579-91A0-6BF106B8465E}" name="HS Jour  ouvrable" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{BF729E3A-D6DD-4796-8AD4-0F6BB601BCEE}" name="HS Jour non ouvrable" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6412,42 +6839,43 @@
   <dimension ref="B2:Q42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7265625" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" customWidth="1"/>
+    <col min="6" max="6" width="14.1796875" customWidth="1"/>
+    <col min="7" max="7" width="11.6328125" customWidth="1"/>
+    <col min="8" max="8" width="14.36328125" customWidth="1"/>
     <col min="11" max="11" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="17.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:17" ht="26" x14ac:dyDescent="0.3">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="36" t="s">
         <v>248</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="65" t="s">
         <v>249</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="66" t="s">
         <v>250</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="66" t="s">
         <v>296</v>
       </c>
-      <c r="F2" s="47" t="s">
+      <c r="F2" s="67" t="s">
         <v>291</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="G2" s="68" t="s">
         <v>288</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="H2" s="69" t="s">
         <v>287</v>
       </c>
       <c r="J2" s="22"/>
-      <c r="N2" s="41" t="s">
+      <c r="N2" s="39" t="s">
         <v>249</v>
       </c>
-      <c r="O2" s="42" t="s">
+      <c r="O2" s="40" t="s">
         <v>248</v>
       </c>
     </row>
@@ -6456,32 +6884,32 @@
         <f t="shared" ref="B3:B33" si="0">TEXT(C3,"jjjj")</f>
         <v>dimanche</v>
       </c>
-      <c r="C3" s="34">
+      <c r="C3" s="63">
         <v>45494</v>
       </c>
-      <c r="D3" s="35">
+      <c r="D3" s="34">
         <v>998</v>
       </c>
-      <c r="E3" s="51">
+      <c r="E3" s="47">
         <v>8</v>
       </c>
       <c r="F3" s="10">
         <f>IF(LEN(TRIM(D3))=2,VLOOKUP(TEXT(D3,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D3,1),"0"),POSE_CSKN,3,0))</f>
         <v>12</v>
       </c>
-      <c r="G3" s="50">
+      <c r="G3" s="46">
         <f>IF(AND(WEEKDAY(C3)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C3)=0),IF(F3&gt;0,F3-IF(WEEKDAY(C3)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="58">
         <f>IF(OR(WEEKDAY(C3)=1,COUNTIF(Tableau_Pose_Cskn[Date],C3)&gt;0),IF(F3&gt;0,F3-IF(WEEKDAY(C3)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
       <c r="I3" s="18"/>
-      <c r="N3" s="43">
+      <c r="N3" s="41">
         <v>45505</v>
       </c>
-      <c r="O3" s="48" t="s">
+      <c r="O3" s="45" t="s">
         <v>290</v>
       </c>
     </row>
@@ -6490,7 +6918,7 @@
         <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="64">
         <v>45495</v>
       </c>
       <c r="D4" s="32">
@@ -6507,15 +6935,15 @@
         <f>IF(AND(WEEKDAY(C4)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C4)=0),IF(F4&gt;0,F4-IF(WEEKDAY(C4)=7,5,8),0),0)</f>
         <v>10</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="58">
         <f>IF(OR(WEEKDAY(C4)=1,COUNTIF(Tableau_Pose_Cskn[Date],C4)&gt;0),IF(F4&gt;0,F4-IF(WEEKDAY(C4)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
       <c r="I4" s="18"/>
-      <c r="N4" s="45">
+      <c r="N4" s="43">
         <v>45651</v>
       </c>
-      <c r="O4" s="46" t="s">
+      <c r="O4" s="44" t="s">
         <v>289</v>
       </c>
     </row>
@@ -6524,13 +6952,13 @@
         <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="64">
         <v>45496</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="52">
+      <c r="E5" s="48">
         <v>8</v>
       </c>
       <c r="F5" s="10">
@@ -6541,7 +6969,7 @@
         <f>IF(AND(WEEKDAY(C5)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C5)=0),IF(F5&gt;0,F5-IF(WEEKDAY(C5)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="58">
         <f>IF(OR(WEEKDAY(C5)=1,COUNTIF(Tableau_Pose_Cskn[Date],C5)&gt;0),IF(F5&gt;0,F5-IF(WEEKDAY(C5)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6552,7 +6980,7 @@
         <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="64">
         <v>45497</v>
       </c>
       <c r="D6" s="32">
@@ -6569,12 +6997,12 @@
         <f>IF(AND(WEEKDAY(C6)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C6)=0),IF(F6&gt;0,F6-IF(WEEKDAY(C6)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="58">
         <f>IF(OR(WEEKDAY(C6)=1,COUNTIF(Tableau_Pose_Cskn[Date],C6)&gt;0),IF(F6&gt;0,F6-IF(WEEKDAY(C6)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
       <c r="I6" s="18"/>
-      <c r="L6" s="44">
+      <c r="L6" s="42">
         <v>45505</v>
       </c>
     </row>
@@ -6583,7 +7011,7 @@
         <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="64">
         <v>45498</v>
       </c>
       <c r="D7" s="32">
@@ -6600,7 +7028,7 @@
         <f>IF(AND(WEEKDAY(C7)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C7)=0),IF(F7&gt;0,F7-IF(WEEKDAY(C7)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="58">
         <f>IF(OR(WEEKDAY(C7)=1,COUNTIF(Tableau_Pose_Cskn[Date],C7)&gt;0),IF(F7&gt;0,F7-IF(WEEKDAY(C7)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6612,7 +7040,7 @@
         <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="64">
         <v>45499</v>
       </c>
       <c r="D8" s="32">
@@ -6629,7 +7057,7 @@
         <f>IF(AND(WEEKDAY(C8)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C8)=0),IF(F8&gt;0,F8-IF(WEEKDAY(C8)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="58">
         <f>IF(OR(WEEKDAY(C8)=1,COUNTIF(Tableau_Pose_Cskn[Date],C8)&gt;0),IF(F8&gt;0,F8-IF(WEEKDAY(C8)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6640,7 +7068,7 @@
         <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="64">
         <v>45500</v>
       </c>
       <c r="D9" s="32">
@@ -6657,7 +7085,7 @@
         <f>IF(AND(WEEKDAY(C9)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C9)=0),IF(F9&gt;0,F9-IF(WEEKDAY(C9)=7,5,8),0),0)</f>
         <v>7</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="58">
         <f>IF(OR(WEEKDAY(C9)=1,COUNTIF(Tableau_Pose_Cskn[Date],C9)&gt;0),IF(F9&gt;0,F9-IF(WEEKDAY(C9)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6669,7 +7097,7 @@
         <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="64">
         <v>45501</v>
       </c>
       <c r="D10" s="32">
@@ -6682,11 +7110,11 @@
         <f>IF(LEN(TRIM(D10))=2,VLOOKUP(TEXT(D10,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D10,1),"0"),POSE_CSKN,3,0))</f>
         <v>12</v>
       </c>
-      <c r="G10" s="50">
+      <c r="G10" s="46">
         <f>IF(AND(WEEKDAY(C10)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C10)=0),IF(F10&gt;0,F10-IF(WEEKDAY(C10)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="58">
         <f>IF(OR(WEEKDAY(C10)=1,COUNTIF(Tableau_Pose_Cskn[Date],C10)&gt;0),IF(F10&gt;0,F10-IF(WEEKDAY(C10)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
@@ -6697,7 +7125,7 @@
         <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="64">
         <v>45502</v>
       </c>
       <c r="D11" s="32">
@@ -6714,7 +7142,7 @@
         <f>IF(AND(WEEKDAY(C11)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C11)=0),IF(F11&gt;0,F11-IF(WEEKDAY(C11)=7,5,8),0),0)</f>
         <v>10</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="58">
         <f>IF(OR(WEEKDAY(C11)=1,COUNTIF(Tableau_Pose_Cskn[Date],C11)&gt;0),IF(F11&gt;0,F11-IF(WEEKDAY(C11)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6725,7 +7153,7 @@
         <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="64">
         <v>45503</v>
       </c>
       <c r="D12" s="32">
@@ -6742,7 +7170,7 @@
         <f>IF(AND(WEEKDAY(C12)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C12)=0),IF(F12&gt;0,F12-IF(WEEKDAY(C12)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="58">
         <f>IF(OR(WEEKDAY(C12)=1,COUNTIF(Tableau_Pose_Cskn[Date],C12)&gt;0),IF(F12&gt;0,F12-IF(WEEKDAY(C12)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6759,7 +7187,7 @@
         <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="64">
         <v>45504</v>
       </c>
       <c r="D13" s="32">
@@ -6776,7 +7204,7 @@
         <f>IF(AND(WEEKDAY(C13)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C13)=0),IF(F13&gt;0,F13-IF(WEEKDAY(C13)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="58">
         <f>IF(OR(WEEKDAY(C13)=1,COUNTIF(Tableau_Pose_Cskn[Date],C13)&gt;0),IF(F13&gt;0,F13-IF(WEEKDAY(C13)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6793,7 +7221,7 @@
         <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="64">
         <v>45505</v>
       </c>
       <c r="D14" s="32">
@@ -6806,11 +7234,11 @@
         <f>IF(LEN(TRIM(D14))=2,VLOOKUP(TEXT(D14,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D14,1),"0"),POSE_CSKN,3,0))</f>
         <v>12</v>
       </c>
-      <c r="G14" s="50">
+      <c r="G14" s="46">
         <f>IF(AND(WEEKDAY(C14)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C14)=0),IF(F14&gt;0,F14-IF(WEEKDAY(C14)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="58">
         <f>IF(OR(WEEKDAY(C14)=1,COUNTIF(Tableau_Pose_Cskn[Date],C14)&gt;0),IF(F14&gt;0,F14-IF(WEEKDAY(C14)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
@@ -6821,7 +7249,7 @@
         <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="64">
         <v>45506</v>
       </c>
       <c r="D15" s="32">
@@ -6838,7 +7266,7 @@
         <f>IF(AND(WEEKDAY(C15)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C15)=0),IF(F15&gt;0,F15-IF(WEEKDAY(C15)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="58">
         <f>IF(OR(WEEKDAY(C15)=1,COUNTIF(Tableau_Pose_Cskn[Date],C15)&gt;0),IF(F15&gt;0,F15-IF(WEEKDAY(C15)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6849,7 +7277,7 @@
         <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="64">
         <v>45507</v>
       </c>
       <c r="D16" s="32">
@@ -6866,7 +7294,7 @@
         <f>IF(AND(WEEKDAY(C16)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C16)=0),IF(F16&gt;0,F16-IF(WEEKDAY(C16)=7,5,8),0),0)</f>
         <v>7</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="58">
         <f>IF(OR(WEEKDAY(C16)=1,COUNTIF(Tableau_Pose_Cskn[Date],C16)&gt;0),IF(F16&gt;0,F16-IF(WEEKDAY(C16)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6877,7 +7305,7 @@
         <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="64">
         <v>45508</v>
       </c>
       <c r="D17" s="32">
@@ -6890,11 +7318,11 @@
         <f>IF(LEN(TRIM(D17))=2,VLOOKUP(TEXT(D17,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D17,1),"0"),POSE_CSKN,3,0))</f>
         <v>12</v>
       </c>
-      <c r="G17" s="50">
+      <c r="G17" s="46">
         <f>IF(AND(WEEKDAY(C17)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C17)=0),IF(F17&gt;0,F17-IF(WEEKDAY(C17)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="58">
         <f>IF(OR(WEEKDAY(C17)=1,COUNTIF(Tableau_Pose_Cskn[Date],C17)&gt;0),IF(F17&gt;0,F17-IF(WEEKDAY(C17)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
@@ -6905,7 +7333,7 @@
         <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="64">
         <v>45509</v>
       </c>
       <c r="D18" s="32">
@@ -6922,7 +7350,7 @@
         <f>IF(AND(WEEKDAY(C18)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C18)=0),IF(F18&gt;0,F18-IF(WEEKDAY(C18)=7,5,8),0),0)</f>
         <v>10</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="58">
         <f>IF(OR(WEEKDAY(C18)=1,COUNTIF(Tableau_Pose_Cskn[Date],C18)&gt;0),IF(F18&gt;0,F18-IF(WEEKDAY(C18)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6933,7 +7361,7 @@
         <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="64">
         <v>45510</v>
       </c>
       <c r="D19" s="32">
@@ -6950,7 +7378,7 @@
         <f>IF(AND(WEEKDAY(C19)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C19)=0),IF(F19&gt;0,F19-IF(WEEKDAY(C19)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="58">
         <f>IF(OR(WEEKDAY(C19)=1,COUNTIF(Tableau_Pose_Cskn[Date],C19)&gt;0),IF(F19&gt;0,F19-IF(WEEKDAY(C19)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6961,7 +7389,7 @@
         <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="64">
         <v>45511</v>
       </c>
       <c r="D20" s="32">
@@ -6978,7 +7406,7 @@
         <f>IF(AND(WEEKDAY(C20)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C20)=0),IF(F20&gt;0,F20-IF(WEEKDAY(C20)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="58">
         <f>IF(OR(WEEKDAY(C20)=1,COUNTIF(Tableau_Pose_Cskn[Date],C20)&gt;0),IF(F20&gt;0,F20-IF(WEEKDAY(C20)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -6989,7 +7417,7 @@
         <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="64">
         <v>45512</v>
       </c>
       <c r="D21" s="32">
@@ -7006,7 +7434,7 @@
         <f>IF(AND(WEEKDAY(C21)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C21)=0),IF(F21&gt;0,F21-IF(WEEKDAY(C21)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="58">
         <f>IF(OR(WEEKDAY(C21)=1,COUNTIF(Tableau_Pose_Cskn[Date],C21)&gt;0),IF(F21&gt;0,F21-IF(WEEKDAY(C21)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7017,7 +7445,7 @@
         <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="64">
         <v>45513</v>
       </c>
       <c r="D22" s="32">
@@ -7034,7 +7462,7 @@
         <f>IF(AND(WEEKDAY(C22)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C22)=0),IF(F22&gt;0,F22-IF(WEEKDAY(C22)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="58">
         <f>IF(OR(WEEKDAY(C22)=1,COUNTIF(Tableau_Pose_Cskn[Date],C22)&gt;0),IF(F22&gt;0,F22-IF(WEEKDAY(C22)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7045,7 +7473,7 @@
         <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="64">
         <v>45514</v>
       </c>
       <c r="D23" s="32">
@@ -7062,7 +7490,7 @@
         <f>IF(AND(WEEKDAY(C23)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C23)=0),IF(F23&gt;0,F23-IF(WEEKDAY(C23)=7,5,8),0),0)</f>
         <v>7</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="58">
         <f>IF(OR(WEEKDAY(C23)=1,COUNTIF(Tableau_Pose_Cskn[Date],C23)&gt;0),IF(F23&gt;0,F23-IF(WEEKDAY(C23)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7073,7 +7501,7 @@
         <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="64">
         <v>45515</v>
       </c>
       <c r="D24" s="32">
@@ -7086,11 +7514,11 @@
         <f>IF(LEN(TRIM(D24))=2,VLOOKUP(TEXT(D24,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D24,1),"0"),POSE_CSKN,3,0))</f>
         <v>12</v>
       </c>
-      <c r="G24" s="50">
+      <c r="G24" s="46">
         <f>IF(AND(WEEKDAY(C24)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C24)=0),IF(F24&gt;0,F24-IF(WEEKDAY(C24)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="58">
         <f>IF(OR(WEEKDAY(C24)=1,COUNTIF(Tableau_Pose_Cskn[Date],C24)&gt;0),IF(F24&gt;0,F24-IF(WEEKDAY(C24)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
@@ -7101,7 +7529,7 @@
         <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="64">
         <v>45516</v>
       </c>
       <c r="D25" s="32">
@@ -7118,7 +7546,7 @@
         <f>IF(AND(WEEKDAY(C25)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C25)=0),IF(F25&gt;0,F25-IF(WEEKDAY(C25)=7,5,8),0),0)</f>
         <v>10</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="58">
         <f>IF(OR(WEEKDAY(C25)=1,COUNTIF(Tableau_Pose_Cskn[Date],C25)&gt;0),IF(F25&gt;0,F25-IF(WEEKDAY(C25)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7129,7 +7557,7 @@
         <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="64">
         <v>45517</v>
       </c>
       <c r="D26" s="32">
@@ -7146,7 +7574,7 @@
         <f>IF(AND(WEEKDAY(C26)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C26)=0),IF(F26&gt;0,F26-IF(WEEKDAY(C26)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="58">
         <f>IF(OR(WEEKDAY(C26)=1,COUNTIF(Tableau_Pose_Cskn[Date],C26)&gt;0),IF(F26&gt;0,F26-IF(WEEKDAY(C26)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7157,7 +7585,7 @@
         <f t="shared" si="0"/>
         <v>mercredi</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="64">
         <v>45518</v>
       </c>
       <c r="D27" s="32">
@@ -7174,7 +7602,7 @@
         <f>IF(AND(WEEKDAY(C27)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C27)=0),IF(F27&gt;0,F27-IF(WEEKDAY(C27)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="58">
         <f>IF(OR(WEEKDAY(C27)=1,COUNTIF(Tableau_Pose_Cskn[Date],C27)&gt;0),IF(F27&gt;0,F27-IF(WEEKDAY(C27)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7185,7 +7613,7 @@
         <f t="shared" si="0"/>
         <v>jeudi</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C28" s="64">
         <v>45519</v>
       </c>
       <c r="D28" s="32">
@@ -7202,7 +7630,7 @@
         <f>IF(AND(WEEKDAY(C28)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C28)=0),IF(F28&gt;0,F28-IF(WEEKDAY(C28)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H28" s="10">
+      <c r="H28" s="58">
         <f>IF(OR(WEEKDAY(C28)=1,COUNTIF(Tableau_Pose_Cskn[Date],C28)&gt;0),IF(F28&gt;0,F28-IF(WEEKDAY(C28)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7213,7 +7641,7 @@
         <f t="shared" si="0"/>
         <v>vendredi</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C29" s="64">
         <v>45520</v>
       </c>
       <c r="D29" s="32">
@@ -7230,7 +7658,7 @@
         <f>IF(AND(WEEKDAY(C29)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C29)=0),IF(F29&gt;0,F29-IF(WEEKDAY(C29)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H29" s="58">
         <f>IF(OR(WEEKDAY(C29)=1,COUNTIF(Tableau_Pose_Cskn[Date],C29)&gt;0),IF(F29&gt;0,F29-IF(WEEKDAY(C29)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7241,7 +7669,7 @@
         <f t="shared" si="0"/>
         <v>samedi</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C30" s="64">
         <v>45521</v>
       </c>
       <c r="D30" s="32">
@@ -7258,7 +7686,7 @@
         <f>IF(AND(WEEKDAY(C30)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C30)=0),IF(F30&gt;0,F30-IF(WEEKDAY(C30)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H30" s="58">
         <f>IF(OR(WEEKDAY(C30)=1,COUNTIF(Tableau_Pose_Cskn[Date],C30)&gt;0),IF(F30&gt;0,F30-IF(WEEKDAY(C30)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7269,7 +7697,7 @@
         <f t="shared" si="0"/>
         <v>dimanche</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C31" s="64">
         <v>45522</v>
       </c>
       <c r="D31" s="32">
@@ -7282,11 +7710,11 @@
         <f>IF(LEN(TRIM(D31))=2,VLOOKUP(TEXT(D31,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D31,1),"0"),POSE_CSKN,3,0))</f>
         <v>12</v>
       </c>
-      <c r="G31" s="50">
+      <c r="G31" s="46">
         <f>IF(AND(WEEKDAY(C31)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C31)=0),IF(F31&gt;0,F31-IF(WEEKDAY(C31)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H31" s="10">
+      <c r="H31" s="58">
         <f>IF(OR(WEEKDAY(C31)=1,COUNTIF(Tableau_Pose_Cskn[Date],C31)&gt;0),IF(F31&gt;0,F31-IF(WEEKDAY(C31)=7,5,8),0),0)</f>
         <v>4</v>
       </c>
@@ -7297,7 +7725,7 @@
         <f t="shared" si="0"/>
         <v>lundi</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C32" s="64">
         <v>45523</v>
       </c>
       <c r="D32" s="32">
@@ -7314,7 +7742,7 @@
         <f>IF(AND(WEEKDAY(C32)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C32)=0),IF(F32&gt;0,F32-IF(WEEKDAY(C32)=7,5,8),0),0)</f>
         <v>10</v>
       </c>
-      <c r="H32" s="10">
+      <c r="H32" s="58">
         <f>IF(OR(WEEKDAY(C32)=1,COUNTIF(Tableau_Pose_Cskn[Date],C32)&gt;0),IF(F32&gt;0,F32-IF(WEEKDAY(C32)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
@@ -7325,39 +7753,39 @@
         <f t="shared" si="0"/>
         <v>mardi</v>
       </c>
-      <c r="C33" s="2">
+      <c r="C33" s="41">
         <v>45524</v>
       </c>
-      <c r="D33" s="39" t="s">
+      <c r="D33" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="E33" s="52">
-        <v>8</v>
-      </c>
-      <c r="F33" s="10">
+      <c r="E33" s="71">
+        <v>8</v>
+      </c>
+      <c r="F33" s="61">
         <f>IF(LEN(TRIM(D33))=2,VLOOKUP(TEXT(D33,"00"),Configurations!$B$5:$G$100,6,0),VLOOKUP(TEXT(RIGHT(D33,1),"0"),POSE_CSKN,3,0))</f>
         <v>0</v>
       </c>
-      <c r="G33" s="10">
+      <c r="G33" s="61">
         <f>IF(AND(WEEKDAY(C33)&gt;1,COUNTIF(Tableau_Pose_Cskn[Date],C33)=0),IF(F33&gt;0,F33-IF(WEEKDAY(C33)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
-      <c r="H33" s="10">
+      <c r="H33" s="53">
         <f>IF(OR(WEEKDAY(C33)=1,COUNTIF(Tableau_Pose_Cskn[Date],C33)&gt;0),IF(F33&gt;0,F33-IF(WEEKDAY(C33)=7,5,8),0),0)</f>
         <v>0</v>
       </c>
       <c r="I33" s="18"/>
     </row>
     <row r="34" spans="2:9" ht="13" x14ac:dyDescent="0.3">
-      <c r="F34" s="36">
+      <c r="F34" s="35">
         <f t="shared" ref="F34:H34" si="1">SUM(F3:F33)</f>
         <v>354</v>
       </c>
-      <c r="G34" s="36">
+      <c r="G34" s="35">
         <f t="shared" si="1"/>
         <v>123</v>
       </c>
-      <c r="H34" s="36">
+      <c r="H34" s="35">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -7372,19 +7800,27 @@
       <c r="E36" s="25">
         <v>2</v>
       </c>
+      <c r="F36" s="62" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="24" t="s">
         <v>259</v>
       </c>
       <c r="C37" s="10">
+        <f>MIN(6,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F37,TB_Prestattion[Date],"&lt;" &amp; F37 + 6))</f>
         <v>6</v>
       </c>
       <c r="D37" s="10">
+        <f>MAX(0,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F37,TB_Prestattion[Date],"&lt;" &amp; F37 + 6) - C37)</f>
         <v>23</v>
       </c>
       <c r="E37" s="10">
         <v>0</v>
+      </c>
+      <c r="F37" s="49">
+        <v>45495</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
@@ -7392,13 +7828,18 @@
         <v>260</v>
       </c>
       <c r="C38" s="10">
+        <f>MIN(6,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F38,TB_Prestattion[Date],"&lt;" &amp; F38 + 6))</f>
         <v>6</v>
       </c>
       <c r="D38" s="10">
+        <f>MAX(0,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F38,TB_Prestattion[Date],"&lt;" &amp; F38 + 6) - C38)</f>
         <v>23</v>
       </c>
       <c r="E38" s="10">
         <v>0</v>
+      </c>
+      <c r="F38" s="49">
+        <v>45502</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
@@ -7406,13 +7847,18 @@
         <v>261</v>
       </c>
       <c r="C39" s="10">
+        <f>MIN(6,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F39,TB_Prestattion[Date],"&lt;" &amp; F39 + 6))</f>
         <v>6</v>
       </c>
-      <c r="D39" s="26">
+      <c r="D39" s="10">
+        <f>MAX(0,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F39,TB_Prestattion[Date],"&lt;" &amp; F39 + 6) - C39)</f>
         <v>23</v>
       </c>
       <c r="E39" s="10">
         <v>0</v>
+      </c>
+      <c r="F39" s="49">
+        <v>45509</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
@@ -7420,13 +7866,18 @@
         <v>262</v>
       </c>
       <c r="C40" s="10">
+        <f>MIN(6,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F40,TB_Prestattion[Date],"&lt;" &amp; F40 + 6))</f>
         <v>6</v>
       </c>
-      <c r="D40" s="26">
+      <c r="D40" s="10">
+        <f>MAX(0,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F40,TB_Prestattion[Date],"&lt;" &amp; F40 + 6) - C40)</f>
         <v>20</v>
       </c>
       <c r="E40" s="10">
         <v>0</v>
+      </c>
+      <c r="F40" s="49">
+        <v>45516</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
@@ -7434,17 +7885,22 @@
         <v>275</v>
       </c>
       <c r="C41" s="10">
+        <f>MIN(6,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F41,TB_Prestattion[Date],"&lt;" &amp; F41 + 6))</f>
         <v>6</v>
       </c>
-      <c r="D41" s="26">
+      <c r="D41" s="10">
+        <f>MAX(0,SUMIFS(TB_Prestattion[HS Jr  ouvré],TB_Prestattion[Date],"&gt;=" &amp; F41,TB_Prestattion[Date],"&lt;" &amp; F41 + 6) - C41)</f>
         <v>4</v>
       </c>
       <c r="E41" s="10">
         <v>0</v>
       </c>
+      <c r="F41" s="49">
+        <v>45523</v>
+      </c>
     </row>
     <row r="42" spans="2:9" ht="13" x14ac:dyDescent="0.3">
-      <c r="B42" s="40" t="s">
+      <c r="B42" s="38" t="s">
         <v>287</v>
       </c>
       <c r="C42" s="10">
@@ -7454,19 +7910,751 @@
         <v>0</v>
       </c>
       <c r="E42" s="10">
+        <f>SUM(TB_Prestattion[HS Jr non ouvré])</f>
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7D5A016-83DC-4051-A8AE-E143FEECBE47}">
+  <dimension ref="A1:P49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
+    <col min="4" max="4" width="21.54296875" customWidth="1"/>
+    <col min="7" max="7" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
+        <v>248</v>
+      </c>
+      <c r="B1" s="59" t="s">
+        <v>249</v>
+      </c>
+      <c r="C1" s="59" t="s">
+        <v>304</v>
+      </c>
+      <c r="D1" s="40" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="B2" s="49">
+        <v>45494</v>
+      </c>
+      <c r="C2" s="10">
+        <v>0</v>
+      </c>
+      <c r="D2" s="58">
+        <v>4</v>
+      </c>
+      <c r="F2" s="42">
+        <v>45495</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>310</v>
+      </c>
+      <c r="I2" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="K2" s="55" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="B3" s="56">
+        <v>45495</v>
+      </c>
+      <c r="C3" s="10">
+        <v>10</v>
+      </c>
+      <c r="D3" s="58">
+        <v>0</v>
+      </c>
+      <c r="G3" s="24" t="s">
+        <v>259</v>
+      </c>
+      <c r="H3" s="10">
+        <f>MIN(6,SUMIFS($C$3:$C$32,$B$3:$B$32,"&gt;="&amp;K3,$B$3:$B$32,"&lt;"&amp;K3+6))</f>
+        <v>6</v>
+      </c>
+      <c r="I3" s="10">
+        <f>MAX(0,SUMIFS(Tableau_Prestation[HS Jour  ouvrable],Tableau_Prestation[Date],"&gt;=" &amp; K3,Tableau_Prestation[Date],"&lt;" &amp; K3 + 6) - H3)</f>
+        <v>23</v>
+      </c>
+      <c r="J3" s="10">
+        <v>0</v>
+      </c>
+      <c r="K3" s="42">
+        <v>45495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="57" t="s">
+        <v>299</v>
+      </c>
+      <c r="B4" s="49">
+        <v>45496</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0</v>
+      </c>
+      <c r="D4" s="58">
+        <v>0</v>
+      </c>
+      <c r="G4" s="24" t="s">
+        <v>260</v>
+      </c>
+      <c r="H4" s="10">
+        <f t="shared" ref="H4:H7" si="0">MIN(6,SUMIFS($C$3:$C$32,$B$3:$B$32,"&gt;="&amp;K4,$B$3:$B$32,"&lt;"&amp;K4+6))</f>
+        <v>6</v>
+      </c>
+      <c r="I4" s="10">
+        <f>MAX(0,SUMIFS(Tableau_Prestation[HS Jour  ouvrable],Tableau_Prestation[Date],"&gt;=" &amp; K4,Tableau_Prestation[Date],"&lt;" &amp; K4 + 6) - H4)</f>
+        <v>23</v>
+      </c>
+      <c r="J4" s="10">
+        <v>0</v>
+      </c>
+      <c r="K4" s="49">
+        <v>45502</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="57" t="s">
+        <v>300</v>
+      </c>
+      <c r="B5" s="49">
+        <v>45497</v>
+      </c>
+      <c r="C5" s="10">
+        <v>4</v>
+      </c>
+      <c r="D5" s="58">
+        <v>0</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>261</v>
+      </c>
+      <c r="H5" s="10">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="I5" s="10">
+        <f>MAX(0,SUMIFS(Tableau_Prestation[HS Jour  ouvrable],Tableau_Prestation[Date],"&gt;=" &amp; K5,Tableau_Prestation[Date],"&lt;" &amp; K5 + 6) - H5)</f>
+        <v>23</v>
+      </c>
+      <c r="J5" s="10">
+        <v>0</v>
+      </c>
+      <c r="K5" s="49">
+        <v>45509</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="57" t="s">
+        <v>301</v>
+      </c>
+      <c r="B6" s="49">
+        <v>45498</v>
+      </c>
+      <c r="C6" s="10">
+        <v>4</v>
+      </c>
+      <c r="D6" s="58">
+        <v>0</v>
+      </c>
+      <c r="G6" s="24" t="s">
+        <v>262</v>
+      </c>
+      <c r="H6" s="10">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="I6" s="10">
+        <f>MAX(0,SUMIFS(Tableau_Prestation[HS Jour  ouvrable],Tableau_Prestation[Date],"&gt;=" &amp; K6,Tableau_Prestation[Date],"&lt;" &amp; K6 + 6) - H6)</f>
+        <v>20</v>
+      </c>
+      <c r="J6" s="10">
+        <v>0</v>
+      </c>
+      <c r="K6" s="49">
+        <v>45516</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="57" t="s">
+        <v>302</v>
+      </c>
+      <c r="B7" s="49">
+        <v>45499</v>
+      </c>
+      <c r="C7" s="10">
+        <v>4</v>
+      </c>
+      <c r="D7" s="58">
+        <v>0</v>
+      </c>
+      <c r="G7" s="24" t="s">
+        <v>275</v>
+      </c>
+      <c r="H7" s="10">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="I7" s="10">
+        <f>MAX(0,SUMIFS(Tableau_Prestation[HS Jour  ouvrable],Tableau_Prestation[Date],"&gt;=" &amp; K7,Tableau_Prestation[Date],"&lt;" &amp; K7 + 6) - H7)</f>
+        <v>4</v>
+      </c>
+      <c r="J7" s="10">
+        <v>0</v>
+      </c>
+      <c r="K7" s="49">
+        <v>45523</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="A8" s="57" t="s">
+        <v>303</v>
+      </c>
+      <c r="B8" s="49">
+        <v>45500</v>
+      </c>
+      <c r="C8" s="10">
+        <v>7</v>
+      </c>
+      <c r="D8" s="58">
+        <v>0</v>
+      </c>
+      <c r="G8" s="38" t="s">
+        <v>307</v>
+      </c>
+      <c r="H8" s="10">
+        <v>0</v>
+      </c>
+      <c r="I8" s="26">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10">
+        <f>SUM(Tableau_Prestation[HS Jour non ouvrable])</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="B9" s="49">
+        <v>45501</v>
+      </c>
+      <c r="C9" s="10">
+        <v>0</v>
+      </c>
+      <c r="D9" s="58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="B10" s="56">
+        <v>45502</v>
+      </c>
+      <c r="C10" s="10">
+        <v>10</v>
+      </c>
+      <c r="D10" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="57" t="s">
+        <v>299</v>
+      </c>
+      <c r="B11" s="49">
+        <v>45503</v>
+      </c>
+      <c r="C11" s="10">
+        <v>4</v>
+      </c>
+      <c r="D11" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="57" t="s">
+        <v>300</v>
+      </c>
+      <c r="B12" s="49">
+        <v>45504</v>
+      </c>
+      <c r="C12" s="10">
+        <v>4</v>
+      </c>
+      <c r="D12" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="57" t="s">
+        <v>301</v>
+      </c>
+      <c r="B13" s="49">
+        <v>45505</v>
+      </c>
+      <c r="C13" s="10">
+        <v>0</v>
+      </c>
+      <c r="D13" s="58">
+        <v>4</v>
+      </c>
+      <c r="L13" s="42">
+        <v>46154</v>
+      </c>
+      <c r="N13" s="42">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="57" t="s">
+        <v>302</v>
+      </c>
+      <c r="B14" s="49">
+        <v>45506</v>
+      </c>
+      <c r="C14" s="10">
+        <v>4</v>
+      </c>
+      <c r="D14" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="57" t="s">
+        <v>303</v>
+      </c>
+      <c r="B15" s="49">
+        <v>45507</v>
+      </c>
+      <c r="C15" s="10">
+        <v>7</v>
+      </c>
+      <c r="D15" s="58">
+        <v>0</v>
+      </c>
+      <c r="L15" t="b">
+        <f>L13&lt;=N13</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="B16" s="49">
+        <v>45508</v>
+      </c>
+      <c r="C16" s="10">
+        <v>0</v>
+      </c>
+      <c r="D16" s="58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="B17" s="56">
+        <v>45509</v>
+      </c>
+      <c r="C17" s="10">
+        <v>10</v>
+      </c>
+      <c r="D17" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="57" t="s">
+        <v>299</v>
+      </c>
+      <c r="B18" s="49">
+        <v>45510</v>
+      </c>
+      <c r="C18" s="10">
+        <v>0</v>
+      </c>
+      <c r="D18" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="57" t="s">
+        <v>300</v>
+      </c>
+      <c r="B19" s="49">
+        <v>45511</v>
+      </c>
+      <c r="C19" s="10">
+        <v>4</v>
+      </c>
+      <c r="D19" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="57" t="s">
+        <v>301</v>
+      </c>
+      <c r="B20" s="49">
+        <v>45512</v>
+      </c>
+      <c r="C20" s="10">
+        <v>4</v>
+      </c>
+      <c r="D20" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="57" t="s">
+        <v>302</v>
+      </c>
+      <c r="B21" s="49">
+        <v>45513</v>
+      </c>
+      <c r="C21" s="10">
+        <v>4</v>
+      </c>
+      <c r="D21" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="57" t="s">
+        <v>303</v>
+      </c>
+      <c r="B22" s="49">
+        <v>45514</v>
+      </c>
+      <c r="C22" s="10">
+        <v>7</v>
+      </c>
+      <c r="D22" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="B23" s="49">
+        <v>45515</v>
+      </c>
+      <c r="C23" s="10">
+        <v>0</v>
+      </c>
+      <c r="D23" s="58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="B24" s="56">
+        <v>45516</v>
+      </c>
+      <c r="C24" s="10">
+        <v>10</v>
+      </c>
+      <c r="D24" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="57" t="s">
+        <v>299</v>
+      </c>
+      <c r="B25" s="49">
+        <v>45517</v>
+      </c>
+      <c r="C25" s="10">
+        <v>4</v>
+      </c>
+      <c r="D25" s="58">
+        <v>0</v>
+      </c>
+      <c r="P25" s="42"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="57" t="s">
+        <v>300</v>
+      </c>
+      <c r="B26" s="49">
+        <v>45518</v>
+      </c>
+      <c r="C26" s="10">
+        <v>4</v>
+      </c>
+      <c r="D26" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="57" t="s">
+        <v>301</v>
+      </c>
+      <c r="B27" s="49">
+        <v>45519</v>
+      </c>
+      <c r="C27" s="10">
+        <v>4</v>
+      </c>
+      <c r="D27" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="57" t="s">
+        <v>302</v>
+      </c>
+      <c r="B28" s="49">
+        <v>45520</v>
+      </c>
+      <c r="C28" s="10">
+        <v>4</v>
+      </c>
+      <c r="D28" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="57" t="s">
+        <v>303</v>
+      </c>
+      <c r="B29" s="49">
+        <v>45521</v>
+      </c>
+      <c r="C29" s="10">
+        <v>0</v>
+      </c>
+      <c r="D29" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="B30" s="49">
+        <v>45522</v>
+      </c>
+      <c r="C30" s="10">
+        <v>0</v>
+      </c>
+      <c r="D30" s="58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="B31" s="56">
+        <v>45523</v>
+      </c>
+      <c r="C31" s="10">
+        <v>10</v>
+      </c>
+      <c r="D31" s="58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="54" t="s">
+        <v>299</v>
+      </c>
+      <c r="B32" s="60">
+        <v>45524</v>
+      </c>
+      <c r="C32" s="61">
+        <v>0</v>
+      </c>
+      <c r="D32" s="53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10">
+        <v>123</v>
+      </c>
+      <c r="D34" s="10">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="50"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="B37" s="49">
+        <v>45505</v>
+      </c>
+      <c r="C37" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="51" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="51" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="51"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="51"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B43" s="25">
+        <v>1.3</v>
+      </c>
+      <c r="C43" s="25">
+        <v>1.6</v>
+      </c>
+      <c r="D43" s="25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="24" t="s">
+        <v>259</v>
+      </c>
+      <c r="B44" s="10">
+        <v>6</v>
+      </c>
+      <c r="C44" s="10">
+        <v>23</v>
+      </c>
+      <c r="D44" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="24" t="s">
+        <v>260</v>
+      </c>
+      <c r="B45" s="10">
+        <v>6</v>
+      </c>
+      <c r="C45" s="10">
+        <v>23</v>
+      </c>
+      <c r="D45" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="24" t="s">
+        <v>261</v>
+      </c>
+      <c r="B46" s="10">
+        <v>6</v>
+      </c>
+      <c r="C46" s="26">
+        <v>23</v>
+      </c>
+      <c r="D46" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="24" t="s">
+        <v>262</v>
+      </c>
+      <c r="B47" s="10">
+        <v>6</v>
+      </c>
+      <c r="C47" s="26">
+        <v>20</v>
+      </c>
+      <c r="D47" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="24" t="s">
+        <v>275</v>
+      </c>
+      <c r="B48" s="10">
+        <v>6</v>
+      </c>
+      <c r="C48" s="26">
+        <v>4</v>
+      </c>
+      <c r="D48" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="13" x14ac:dyDescent="0.3">
+      <c r="A49" s="38" t="s">
+        <v>307</v>
+      </c>
+      <c r="B49" s="10">
+        <v>0</v>
+      </c>
+      <c r="C49" s="26">
+        <v>0</v>
+      </c>
+      <c r="D49" s="10">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C4B13EC-8B82-40DB-83EF-CA61C09CB06B}">
   <dimension ref="B2:E49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -7494,7 +8682,7 @@
       <c r="B3" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="C3" s="53">
+      <c r="C3" s="49">
         <v>45494</v>
       </c>
       <c r="D3" s="10">
@@ -7508,7 +8696,7 @@
       <c r="B4" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="C4" s="53">
+      <c r="C4" s="49">
         <v>45495</v>
       </c>
       <c r="D4" s="10">
@@ -7522,7 +8710,7 @@
       <c r="B5" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="C5" s="53">
+      <c r="C5" s="49">
         <v>45496</v>
       </c>
       <c r="D5" s="10">
@@ -7536,7 +8724,7 @@
       <c r="B6" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C6" s="53">
+      <c r="C6" s="49">
         <v>45497</v>
       </c>
       <c r="D6" s="10">
@@ -7550,7 +8738,7 @@
       <c r="B7" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="C7" s="53">
+      <c r="C7" s="49">
         <v>45498</v>
       </c>
       <c r="D7" s="10">
@@ -7564,7 +8752,7 @@
       <c r="B8" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="C8" s="53">
+      <c r="C8" s="49">
         <v>45499</v>
       </c>
       <c r="D8" s="10">
@@ -7578,7 +8766,7 @@
       <c r="B9" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C9" s="53">
+      <c r="C9" s="49">
         <v>45500</v>
       </c>
       <c r="D9" s="10">
@@ -7592,7 +8780,7 @@
       <c r="B10" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="49">
         <v>45501</v>
       </c>
       <c r="D10" s="10">
@@ -7606,7 +8794,7 @@
       <c r="B11" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="C11" s="53">
+      <c r="C11" s="49">
         <v>45502</v>
       </c>
       <c r="D11" s="10">
@@ -7620,7 +8808,7 @@
       <c r="B12" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="C12" s="53">
+      <c r="C12" s="49">
         <v>45503</v>
       </c>
       <c r="D12" s="10">
@@ -7634,7 +8822,7 @@
       <c r="B13" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C13" s="53">
+      <c r="C13" s="49">
         <v>45504</v>
       </c>
       <c r="D13" s="10">
@@ -7648,7 +8836,7 @@
       <c r="B14" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="C14" s="53">
+      <c r="C14" s="49">
         <v>45505</v>
       </c>
       <c r="D14" s="10">
@@ -7662,7 +8850,7 @@
       <c r="B15" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="C15" s="53">
+      <c r="C15" s="49">
         <v>45506</v>
       </c>
       <c r="D15" s="10">
@@ -7676,7 +8864,7 @@
       <c r="B16" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C16" s="53">
+      <c r="C16" s="49">
         <v>45507</v>
       </c>
       <c r="D16" s="10">
@@ -7690,7 +8878,7 @@
       <c r="B17" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="C17" s="53">
+      <c r="C17" s="49">
         <v>45508</v>
       </c>
       <c r="D17" s="10">
@@ -7704,7 +8892,7 @@
       <c r="B18" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="C18" s="53">
+      <c r="C18" s="49">
         <v>45509</v>
       </c>
       <c r="D18" s="10">
@@ -7718,7 +8906,7 @@
       <c r="B19" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="C19" s="53">
+      <c r="C19" s="49">
         <v>45510</v>
       </c>
       <c r="D19" s="10">
@@ -7732,7 +8920,7 @@
       <c r="B20" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C20" s="53">
+      <c r="C20" s="49">
         <v>45511</v>
       </c>
       <c r="D20" s="10">
@@ -7746,7 +8934,7 @@
       <c r="B21" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="C21" s="53">
+      <c r="C21" s="49">
         <v>45512</v>
       </c>
       <c r="D21" s="10">
@@ -7760,7 +8948,7 @@
       <c r="B22" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="C22" s="53">
+      <c r="C22" s="49">
         <v>45513</v>
       </c>
       <c r="D22" s="10">
@@ -7774,7 +8962,7 @@
       <c r="B23" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C23" s="53">
+      <c r="C23" s="49">
         <v>45514</v>
       </c>
       <c r="D23" s="10">
@@ -7788,7 +8976,7 @@
       <c r="B24" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="C24" s="53">
+      <c r="C24" s="49">
         <v>45515</v>
       </c>
       <c r="D24" s="10">
@@ -7802,7 +8990,7 @@
       <c r="B25" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="C25" s="53">
+      <c r="C25" s="49">
         <v>45516</v>
       </c>
       <c r="D25" s="10">
@@ -7816,7 +9004,7 @@
       <c r="B26" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="C26" s="53">
+      <c r="C26" s="49">
         <v>45517</v>
       </c>
       <c r="D26" s="10">
@@ -7830,7 +9018,7 @@
       <c r="B27" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C27" s="53">
+      <c r="C27" s="49">
         <v>45518</v>
       </c>
       <c r="D27" s="10">
@@ -7844,7 +9032,7 @@
       <c r="B28" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="C28" s="53">
+      <c r="C28" s="49">
         <v>45519</v>
       </c>
       <c r="D28" s="10">
@@ -7858,7 +9046,7 @@
       <c r="B29" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="C29" s="53">
+      <c r="C29" s="49">
         <v>45520</v>
       </c>
       <c r="D29" s="10">
@@ -7872,7 +9060,7 @@
       <c r="B30" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C30" s="53">
+      <c r="C30" s="49">
         <v>45521</v>
       </c>
       <c r="D30" s="10">
@@ -7886,7 +9074,7 @@
       <c r="B31" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="C31" s="53">
+      <c r="C31" s="49">
         <v>45522</v>
       </c>
       <c r="D31" s="10">
@@ -7900,7 +9088,7 @@
       <c r="B32" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="C32" s="53">
+      <c r="C32" s="49">
         <v>45523</v>
       </c>
       <c r="D32" s="10">
@@ -7914,7 +9102,7 @@
       <c r="B33" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="C33" s="53">
+      <c r="C33" s="49">
         <v>45524</v>
       </c>
       <c r="D33" s="10">
@@ -7935,16 +9123,16 @@
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="54"/>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="C37" s="53">
+      <c r="C37" s="49">
         <v>45505</v>
       </c>
       <c r="D37" t="s">
@@ -7952,20 +9140,20 @@
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B39" s="55" t="s">
+      <c r="B39" s="51" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B40" s="55" t="s">
+      <c r="B40" s="51" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B41" s="55"/>
+      <c r="B41" s="51"/>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B42" s="55"/>
+      <c r="B42" s="51"/>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C43" s="25">
@@ -8049,7 +9237,7 @@
       </c>
     </row>
     <row r="49" spans="2:5" ht="13" x14ac:dyDescent="0.3">
-      <c r="B49" s="40" t="s">
+      <c r="B49" s="38" t="s">
         <v>307</v>
       </c>
       <c r="C49" s="10">
@@ -8068,7 +9256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5287AAF-25F6-426B-93DC-326260F9D879}">
   <dimension ref="B3:M100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -8084,17 +9272,17 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:13" ht="13" x14ac:dyDescent="0.3">
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="52" t="s">
         <v>285</v>
       </c>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="K3" s="49" t="s">
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="K3" s="52" t="s">
         <v>286</v>
       </c>
-      <c r="L3" s="49"/>
-      <c r="M3" s="49"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="52"/>
     </row>
     <row r="5" spans="2:13" ht="26" x14ac:dyDescent="0.25">
       <c r="B5" s="8" t="s">

</xml_diff>